<commit_message>
feat(feishu_bot): enhance SQL generation and session management
- Introduced a new ProcRef class to manage subprocess references for better control over SQL generation processes.
- Updated CursorClient to support unique prompt file naming for concurrent requests, preventing file overwrites.
- Enhanced Workflow class with request versioning to ensure message handling corresponds to the latest user requests, improving user experience.
- Added reset functionality to clear session state, allowing users to start fresh when needed.
- Improved feedback mechanisms during SQL generation and execution phases to keep users informed of progress and actions.
</commit_message>
<xml_diff>
--- a/input/通话Id.xlsx
+++ b/input/通话Id.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14700" windowHeight="8080"/>
+    <workbookView windowWidth="18600" windowHeight="8080"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,2404 +32,2404 @@
     <t>通话id</t>
   </si>
   <si>
-    <t>0037ecba7a0d4c8ea1b7e04afc27fa55</t>
-  </si>
-  <si>
-    <t>014dd345102842bb91145d8357dc43b7</t>
-  </si>
-  <si>
-    <t>018ef8743b664149a4c46626e5d73afa</t>
-  </si>
-  <si>
-    <t>01e8335e1bda4f29982da8c0d10d37c2</t>
-  </si>
-  <si>
-    <t>02381e6eae114ceb92fc4bd41a3750d0</t>
-  </si>
-  <si>
-    <t>0287f584b6f449ac93cc936d6687d9c4</t>
-  </si>
-  <si>
-    <t>02fa29a984c0499daa94689e8bd65b20</t>
-  </si>
-  <si>
-    <t>032fba241a39484cb88ae7a56e28ccc9</t>
-  </si>
-  <si>
-    <t>033237d02b3a4e02a535f08129fa811b</t>
-  </si>
-  <si>
-    <t>033e202d02e24203a3a25737bd32f6e5</t>
-  </si>
-  <si>
-    <t>036f9daa002f4ed197d4daa4dce5b8c1</t>
-  </si>
-  <si>
-    <t>03b01e06903d4e53b4d455ea278c8979</t>
-  </si>
-  <si>
-    <t>03df90d551814cf4ad31fc9dec100a53</t>
-  </si>
-  <si>
-    <t>040d369725e240508a9ab086636b5118</t>
-  </si>
-  <si>
-    <t>041cd424d4924642995be2b2cdf93e6b</t>
-  </si>
-  <si>
-    <t>044f1739782b40c9ae6e8794062c0a25</t>
-  </si>
-  <si>
-    <t>046bb208649842678fc90da3ad8d5b57</t>
-  </si>
-  <si>
-    <t>046c6a385a3b45d693e77aa2bdfbd1af</t>
-  </si>
-  <si>
-    <t>05bd7d00e2c84eb78556102efc197bc8</t>
-  </si>
-  <si>
-    <t>05fcc6f62a83482b84afb7fd594b3e57</t>
-  </si>
-  <si>
-    <t>0627b8e3e7a14f059cb04e1843501b1c</t>
-  </si>
-  <si>
-    <t>068a013670d841d887ce12b7a5556c57</t>
-  </si>
-  <si>
-    <t>06b5935a4d4c4a9391f8195f194301ac</t>
-  </si>
-  <si>
-    <t>06e5dd47944a482c9f25528157026e8d</t>
-  </si>
-  <si>
-    <t>075180f9ee964e5880ca209b77994d58</t>
-  </si>
-  <si>
-    <t>07636b357eb14da2b38834f97137fc67</t>
-  </si>
-  <si>
-    <t>077e18ffe6694b4799860e0b4052e736</t>
-  </si>
-  <si>
-    <t>078d6826840e456bbd950b5fb9186c22</t>
-  </si>
-  <si>
-    <t>07e891fb87584b5693b1747a49941d44</t>
-  </si>
-  <si>
-    <t>0804e11ac6d64f8e8e05f6105d25ca63</t>
-  </si>
-  <si>
-    <t>090534a5db9d4d3287737ec117677ade</t>
-  </si>
-  <si>
-    <t>0977ba4dcc8c43699d8aa49fb9deef04</t>
-  </si>
-  <si>
-    <t>098382dabe9a4e07a0a72dacc88716d2</t>
-  </si>
-  <si>
-    <t>098e717215b847ec84a097312d54c0b0</t>
-  </si>
-  <si>
-    <t>09fd3ea7c7c947e6bde2a9941d85e77d</t>
-  </si>
-  <si>
-    <t>0a59f3ab81e945c4a3fc928272d469e6</t>
-  </si>
-  <si>
-    <t>0c1a7c2d0dc14174a5c38eb33e0956e1</t>
-  </si>
-  <si>
-    <t>0c464dacf02246929ee8ea2766337681</t>
-  </si>
-  <si>
-    <t>0d0741553b4b40ce9c47129f81634296</t>
-  </si>
-  <si>
-    <t>0d546cd90c9641dfa64d5f6c3297649d</t>
-  </si>
-  <si>
-    <t>0d88fc40f26f4fd1a391456c690a50ec</t>
-  </si>
-  <si>
-    <t>0de1c9a0b3ad47de995dc58a3c1afa1a</t>
-  </si>
-  <si>
-    <t>0de830c1e8a545c1b7a8f4cffe87b406</t>
-  </si>
-  <si>
-    <t>0efc86bbfbe94e0f8d36d8ef1194085f</t>
-  </si>
-  <si>
-    <t>0f85d864855f4c2d9faffc8b4929321a</t>
-  </si>
-  <si>
-    <t>0fac61a6d45243c6a9a7c02f9f6488f9</t>
-  </si>
-  <si>
-    <t>0fd91c8692164715b1ea1c87bd50dd6a</t>
-  </si>
-  <si>
-    <t>10202320039e417eabb83776eb1433e8</t>
-  </si>
-  <si>
-    <t>109498f18b0840348204679b342f8bce</t>
-  </si>
-  <si>
-    <t>10cfd918da9a4322afc8115c683a4a23</t>
-  </si>
-  <si>
-    <t>10ee23bb9f544e68af09a2a51d72412e</t>
-  </si>
-  <si>
-    <t>10f7d853cd834bcf9d2a7bfc8466c2ef</t>
-  </si>
-  <si>
-    <t>11124c040b6445708200ecff9ff573d2</t>
-  </si>
-  <si>
-    <t>114665a6c6074f8e90547bc6b56f58e5</t>
-  </si>
-  <si>
-    <t>11c4d61c50eb47a8b3c4eaac2d302278</t>
-  </si>
-  <si>
-    <t>11cfe877ac584a3fb601908c25254236</t>
-  </si>
-  <si>
-    <t>1214eb27b4ac428eb335e45b3c74612a</t>
-  </si>
-  <si>
-    <t>1241a68c56064b2a92e4e1ab67ed04dd</t>
-  </si>
-  <si>
-    <t>1247e2d9be3c48f6975315e9127781b8</t>
-  </si>
-  <si>
-    <t>12be31b9ae5b45de93674c8c9dbc4fff</t>
-  </si>
-  <si>
-    <t>12d26bdfe295427e8a4447b21b32f8bc</t>
-  </si>
-  <si>
-    <t>12d4ce7350f94aa0860c75a9a9a30744</t>
-  </si>
-  <si>
-    <t>12ead5ad55074d08abadd47c0218e49f</t>
-  </si>
-  <si>
-    <t>13724a2551464262a3cb6bb793bb19a7</t>
-  </si>
-  <si>
-    <t>13930806a6154413b7bfa1d6f2eb4fbc</t>
-  </si>
-  <si>
-    <t>1440814da4914220b9aab28c28bfe50a</t>
-  </si>
-  <si>
-    <t>14b564d2f20648b795b6967d2dbe547e</t>
-  </si>
-  <si>
-    <t>15223d7515af4f7dab52bb7873572081</t>
-  </si>
-  <si>
-    <t>15303f73b8c54b27ac94608ae71f854f</t>
-  </si>
-  <si>
-    <t>1535139fe1dc4d4cada78c33add27f73</t>
-  </si>
-  <si>
-    <t>1556782fa7ef4310a16f1625f23ea757</t>
-  </si>
-  <si>
-    <t>155e123f65954cc6bc3328e34b8bf6dc</t>
-  </si>
-  <si>
-    <t>15f3e58b3be54d2bae71035cb2d9c39f</t>
-  </si>
-  <si>
-    <t>1626711b169a420abb8a06d5d70ac632</t>
-  </si>
-  <si>
-    <t>16ab0118a75b42eeabb0bac6ca1e6be8</t>
-  </si>
-  <si>
-    <t>16d756dd76e84975b5f006ddbfa75875</t>
-  </si>
-  <si>
-    <t>177831576563432baf95b3e9909709df</t>
-  </si>
-  <si>
-    <t>17b4f064189f41829e56eee0bf3b8184</t>
-  </si>
-  <si>
-    <t>17bcb05a40d8416ba442d5f958661444</t>
-  </si>
-  <si>
-    <t>17e84703833447a1a2989eef52acc944</t>
-  </si>
-  <si>
-    <t>17f6b99beeb44703adba12bcbd5177af</t>
-  </si>
-  <si>
-    <t>185b5dc26b20421b8fe07ac44d49514c</t>
-  </si>
-  <si>
-    <t>186a5c44391748b08b6692dd98844c05</t>
-  </si>
-  <si>
-    <t>18a7544e205745ce8174b8eda1f670aa</t>
-  </si>
-  <si>
-    <t>194fa4c5f33a4946ae45aaf2629d78e4</t>
-  </si>
-  <si>
-    <t>19734edece424395b29a4b8a4458b487</t>
-  </si>
-  <si>
-    <t>197c49e63ec144b59717dcbb9bd6866c</t>
-  </si>
-  <si>
-    <t>1b1828d543f040a89376b2b044780373</t>
-  </si>
-  <si>
-    <t>1b318b350b9c4e66be75c3ea1432439a</t>
-  </si>
-  <si>
-    <t>1b4fb58cddc04c1487a615d9dc7e9636</t>
-  </si>
-  <si>
-    <t>1b70448ad57048d5a682e7e19506dca3</t>
-  </si>
-  <si>
-    <t>1bfbeb58293f4ec4b06f64871b3aa155</t>
-  </si>
-  <si>
-    <t>1c1e16dc1a9c4959aa914e3003f2b348</t>
-  </si>
-  <si>
-    <t>1c429bebeefe4bedb9d76b4ea0aee05a</t>
-  </si>
-  <si>
-    <t>1c43c7a9d9e8424ebb8a07a26a954ef7</t>
-  </si>
-  <si>
-    <t>1c9db81f0b824705b66e3f63c980b0ba</t>
-  </si>
-  <si>
-    <t>1d01bcc72c5e453d8ab4ba6b22666c04</t>
-  </si>
-  <si>
-    <t>1d1c33ed6a2f4efabb670a597368f414</t>
-  </si>
-  <si>
-    <t>1d43998dcf0b48ba8baa89a485f48826</t>
-  </si>
-  <si>
-    <t>1d4e9be8c9cc4383b987699371b1bb48</t>
-  </si>
-  <si>
-    <t>1dfe7fd95fe941f38c58e0398aeecdc8</t>
-  </si>
-  <si>
-    <t>1e61f7a906574c7b830657d0f42d5814</t>
-  </si>
-  <si>
-    <t>1eef252dc1e9499195009ac3af48e219</t>
-  </si>
-  <si>
-    <t>1f04c0cd26a741748849bd0ae0f3c428</t>
-  </si>
-  <si>
-    <t>1f475a05ce6942248aa7d97bea9d640b</t>
-  </si>
-  <si>
-    <t>1fb2aaeb4a274f6397083aac6162dc9d</t>
-  </si>
-  <si>
-    <t>2038442948024798bfc1ecacba64a0b0</t>
-  </si>
-  <si>
-    <t>2063152b17454d798424420e6d35879e</t>
-  </si>
-  <si>
-    <t>20c47b792a1444039afc1ec03ddf6a5c</t>
-  </si>
-  <si>
-    <t>2189e95254324a29990e2f9c845536a2</t>
-  </si>
-  <si>
-    <t>220f644a7d3240ceb59b3f8f69cc949a</t>
-  </si>
-  <si>
-    <t>222f113e486a48f8aaff7dca11829b5e</t>
-  </si>
-  <si>
-    <t>223400e7f09b4e35b19643ad228c09b0</t>
-  </si>
-  <si>
-    <t>23b3cf416c8f460d8240ab3da47132fe</t>
-  </si>
-  <si>
-    <t>23ec52301af54d3885fc5fb46de1cb68</t>
-  </si>
-  <si>
-    <t>242913cf2ffb42abaa06aa86da3f7020</t>
-  </si>
-  <si>
-    <t>24f4a224a46949f7a370f42720fbf152</t>
-  </si>
-  <si>
-    <t>250de5cc9340470e9bab943fad3d29cc</t>
-  </si>
-  <si>
-    <t>251e8bfb8a8749838faef618eb63f5d8</t>
-  </si>
-  <si>
-    <t>252a0fa5271746ac9b8779b1943a1bb6</t>
-  </si>
-  <si>
-    <t>25591f97c3fc4f21a4512071e5e2ea2d</t>
-  </si>
-  <si>
-    <t>25ff1805c4644024b3bb4181cc6cf9d3</t>
-  </si>
-  <si>
-    <t>26f3652b7b274b3a93f94e6a1cf5d18d</t>
-  </si>
-  <si>
-    <t>271cbf3fc2f54808be583bb31de55909</t>
-  </si>
-  <si>
-    <t>28108450bcd24e409fe7ad206b36e1e7</t>
-  </si>
-  <si>
-    <t>282dcc1f951a444fbcd55d00871fc591</t>
-  </si>
-  <si>
-    <t>285c7d9d6e2746dbaf3952a515292fef</t>
-  </si>
-  <si>
-    <t>287c33f93c114884b2c97ffb1b692fe9</t>
-  </si>
-  <si>
-    <t>28f7e2054c1440f787cf958c05edabe2</t>
-  </si>
-  <si>
-    <t>2949297bae38474fa25bb674ebad0a0f</t>
-  </si>
-  <si>
-    <t>2a817daeb62a4b5cbd808750c796279b</t>
-  </si>
-  <si>
-    <t>2af2079380d947b3b3ee9cef7e1e6399</t>
-  </si>
-  <si>
-    <t>2b16168af7d945c7b4ea126214507bfd</t>
-  </si>
-  <si>
-    <t>2b330ee53c5b401fbc21b6f9196866c9</t>
-  </si>
-  <si>
-    <t>2b6ff5e34d114b31bc3d59bbe0f0e775</t>
-  </si>
-  <si>
-    <t>2b7ace11776e4035ab1f9cdd63297444</t>
-  </si>
-  <si>
-    <t>2bf8f0a8b6a24ee691b39b7007c96bdc</t>
-  </si>
-  <si>
-    <t>2c49bc3b17ba46bc9f07b463ea3f58ec</t>
-  </si>
-  <si>
-    <t>2c4b4893e2ae40beac82e046678ee102</t>
-  </si>
-  <si>
-    <t>2c511d5b303b43838b789c538d22450d</t>
-  </si>
-  <si>
-    <t>2c9340f7a3fd491bafa76f156afc570c</t>
-  </si>
-  <si>
-    <t>2cd5471ed0d049c59e8ac24cd2c954b8</t>
-  </si>
-  <si>
-    <t>2ce657cdb80a45f6a331d9ff29070aa3</t>
-  </si>
-  <si>
-    <t>2d30b529bdc948f99fffec8b5727b794</t>
-  </si>
-  <si>
-    <t>2daaa7328052402a9ec069449b31ed98</t>
-  </si>
-  <si>
-    <t>2df6d2e781924a1f96f9993e25abd9da</t>
-  </si>
-  <si>
-    <t>2e347ed5abe24b37b9e20961968b1e0b</t>
-  </si>
-  <si>
-    <t>2f415930911e401d972afba32c4f5a2f</t>
-  </si>
-  <si>
-    <t>2ff523e4203546458178fcda3c81d0e2</t>
-  </si>
-  <si>
-    <t>301758ad0a9343b6a9b11dcc0d56f4ca</t>
-  </si>
-  <si>
-    <t>3034cf43d6324804937a7da3b44512d0</t>
-  </si>
-  <si>
-    <t>309fdca00f2348e58621de8baa998739</t>
-  </si>
-  <si>
-    <t>30a13e2b67f241fbac713515bdb3a6fb</t>
-  </si>
-  <si>
-    <t>30d37e577b494d45b9b52d63cb836f4d</t>
-  </si>
-  <si>
-    <t>30e2310fe57a4741b63436d2b3c30d95</t>
-  </si>
-  <si>
-    <t>31810a7ebd804e5d96048b0a5d128734</t>
-  </si>
-  <si>
-    <t>31bc60a708b448ccaab3dc42b1a1705a</t>
-  </si>
-  <si>
-    <t>31c769e0e45f430b8c2550635d709697</t>
-  </si>
-  <si>
-    <t>32ce8f9b363a49df96c09fb0b674042f</t>
-  </si>
-  <si>
-    <t>32de733589664c59a0f98442d999d5bb</t>
-  </si>
-  <si>
-    <t>32ffe191fc794735a329ef5f4deb18c6</t>
-  </si>
-  <si>
-    <t>3324a08917884537aebeffa2e7a9b97a</t>
-  </si>
-  <si>
-    <t>339487570aad4fe18130f69a4475c962</t>
-  </si>
-  <si>
-    <t>33f751a7f2f34bf99566b781376f8eba</t>
-  </si>
-  <si>
-    <t>34140d30ccbf4b018b2d1fbd67b2538f</t>
-  </si>
-  <si>
-    <t>3427382a2811469db96156b1d23ebce6</t>
-  </si>
-  <si>
-    <t>342fa05e60d44a5dbc5a923b272b37bc</t>
-  </si>
-  <si>
-    <t>35295d2784b541cb82f1faf674030106</t>
-  </si>
-  <si>
-    <t>3577844f29424932b83f58008a17032a</t>
-  </si>
-  <si>
-    <t>35dd8e95de6e48039cb8c4abb8484839</t>
-  </si>
-  <si>
-    <t>3656b6f00810421192f5c6b46eebdfd9</t>
-  </si>
-  <si>
-    <t>369fd93c0c7e4e22ad290c0562b3b4be</t>
-  </si>
-  <si>
-    <t>370b6018a7d241368c0d7c93e0c526a6</t>
-  </si>
-  <si>
-    <t>373fe5f235bb4097932f45cdf0b8a7c3</t>
-  </si>
-  <si>
-    <t>38c1641e20d14dbc8516726b8ceb3af7</t>
-  </si>
-  <si>
-    <t>38c8f0b4eb674de4bc90a2f546095188</t>
-  </si>
-  <si>
-    <t>395a4840a656487f95c2a54d5a1a13bc</t>
-  </si>
-  <si>
-    <t>39766346fdb3457fa496163e0260bb57</t>
-  </si>
-  <si>
-    <t>399299da12c84f728c8932b36eab6776</t>
-  </si>
-  <si>
-    <t>39abb5995011416e85df12d02d48af86</t>
-  </si>
-  <si>
-    <t>39bbb54fdb194d38acf7287062185606</t>
-  </si>
-  <si>
-    <t>39bdc330c0b84d80b1282e98058ae568</t>
-  </si>
-  <si>
-    <t>39cf5e599ba144fb89834c164790d6d8</t>
-  </si>
-  <si>
-    <t>3ad680ba99bb4310bccf1ad0daf493ad</t>
-  </si>
-  <si>
-    <t>3b1db3623f1c48e987831691486f1adb</t>
-  </si>
-  <si>
-    <t>3b364a3b273847f78dbf8df0dfcbf0ec</t>
-  </si>
-  <si>
-    <t>3bfcd091e6094cad9b299df8c5581aec</t>
-  </si>
-  <si>
-    <t>3bfd1e0e553f4519b5c327f0ad10a554</t>
-  </si>
-  <si>
-    <t>3c28cdc2db244c959e3e37e932ce6e20</t>
-  </si>
-  <si>
-    <t>3c8215e9a680438db211ffc10ba94108</t>
-  </si>
-  <si>
-    <t>3cc8fc364fd34d4ba2f1a6b94a1f94ef</t>
-  </si>
-  <si>
-    <t>3cf3596f878b4bf6a0f61f0148ce4e3d</t>
-  </si>
-  <si>
-    <t>3e17a94951b44aeb9e7d2518da321663</t>
-  </si>
-  <si>
-    <t>3e21545002734b259dc865b87ae79b1f</t>
-  </si>
-  <si>
-    <t>3e49b2ae38fd4331a4c3a85396806d25</t>
-  </si>
-  <si>
-    <t>3e50ea74e7ce45e4aa180d7b4ba0c77c</t>
-  </si>
-  <si>
-    <t>3ed766c43fc548eb85dbd52c049b621a</t>
-  </si>
-  <si>
-    <t>3edf0a76c9ee489eb43a51aeb1586115</t>
-  </si>
-  <si>
-    <t>3f06dd9ab52d43cba65d394a89ff9fe2</t>
-  </si>
-  <si>
-    <t>3f3ab4f645df4d5e8f84620bc93f2cc8</t>
-  </si>
-  <si>
-    <t>3f53942addbd43bcb0b9057a008b1b6c</t>
-  </si>
-  <si>
-    <t>3f5d4628575f4017b8b9bdd17891832a</t>
-  </si>
-  <si>
-    <t>3f7ce236f92d46cb890a973de6ce48a0</t>
-  </si>
-  <si>
-    <t>3f94b21bc579407487703b12c2175ad3</t>
-  </si>
-  <si>
-    <t>3fdca5357830499da49f1a033b8f9392</t>
-  </si>
-  <si>
-    <t>40a12afa17184a939a5e22345de822c9</t>
-  </si>
-  <si>
-    <t>40ade00fe5bc44fab813342df0ee7cc4</t>
-  </si>
-  <si>
-    <t>40ce0fcdc55a48b2bd1b94503cddf861</t>
-  </si>
-  <si>
-    <t>410caf055b1a4ce8bec493615245876b</t>
-  </si>
-  <si>
-    <t>41283a65e72a4aa4b8b1878f0fbdcf3a</t>
-  </si>
-  <si>
-    <t>415cb74af1934086a39377de9ce89450</t>
-  </si>
-  <si>
-    <t>42545a5b0e3344eabd0d742f53c2e51f</t>
-  </si>
-  <si>
-    <t>425a6df5e60b40889a609b925006a7a8</t>
-  </si>
-  <si>
-    <t>428c9171fe224ffd846afabe15149848</t>
-  </si>
-  <si>
-    <t>429569ab910a4e10866b4489d00d2ee2</t>
-  </si>
-  <si>
-    <t>42c5ed6273c444e9af16af9db8d0d2d5</t>
-  </si>
-  <si>
-    <t>4345acc17a524a50a09eb7e4cc5f6b21</t>
-  </si>
-  <si>
-    <t>43a1d527abfd4b36ad483bed1209d8f5</t>
-  </si>
-  <si>
-    <t>43e3264e7e35435ca12796be01071e2e</t>
-  </si>
-  <si>
-    <t>43fb2b562ff0459d8e5ece3ee54023ef</t>
-  </si>
-  <si>
-    <t>442f7a266ee24b31a368153de49ebf0e</t>
-  </si>
-  <si>
-    <t>4470ab6bd85a43cb9932eec19eb25be0</t>
-  </si>
-  <si>
-    <t>4484e652eab44cd1ac7f2c1d2d6f1111</t>
-  </si>
-  <si>
-    <t>44c18826c0e442759a9435c16b1c438b</t>
-  </si>
-  <si>
-    <t>451411bb655a41fa80e844366767b57d</t>
-  </si>
-  <si>
-    <t>451b6fee013548b2abbff6e35add4ac2</t>
-  </si>
-  <si>
-    <t>4551d22d68ef4fea9038a14c4f38b90e</t>
-  </si>
-  <si>
-    <t>455fabfc075a408bb55abd3777c0fda1</t>
-  </si>
-  <si>
-    <t>45787b56ffe44c91bad4df5f055b70d8</t>
-  </si>
-  <si>
-    <t>45aab857d73c4117a44cd6095e3c3a0d</t>
-  </si>
-  <si>
-    <t>45d60dac70124f75a3e232029c5a4cbd</t>
-  </si>
-  <si>
-    <t>462f664185ed43a494c0dc4c6c652070</t>
-  </si>
-  <si>
-    <t>46a0585216bd42bfb153530df4cae891</t>
-  </si>
-  <si>
-    <t>481aabb006f34e00b251858434415a3a</t>
-  </si>
-  <si>
-    <t>481e96fa9ac54bd3a1a4aec7c4c0cad7</t>
-  </si>
-  <si>
-    <t>484040be64b54999ae446f2c66f67577</t>
-  </si>
-  <si>
-    <t>487c6b755e8f4e5bb8eb486b622240be</t>
-  </si>
-  <si>
-    <t>48c67f6feb4742f09468cca7c4a28f9a</t>
-  </si>
-  <si>
-    <t>4a4d9c390e2946cd87c004abda1f7590</t>
-  </si>
-  <si>
-    <t>4b1afbc0e25f4ad7b4d48ea86c26a180</t>
-  </si>
-  <si>
-    <t>4b1b45e915f3464db077729d0c9fd525</t>
-  </si>
-  <si>
-    <t>4b1d87afe5df4183af4703421252319f</t>
-  </si>
-  <si>
-    <t>4b4322497da6422090b72d320524e171</t>
-  </si>
-  <si>
-    <t>4b4b7a89c7594337b66a64299ff94467</t>
-  </si>
-  <si>
-    <t>4c4016560f224c618a9d1f9b614a440f</t>
-  </si>
-  <si>
-    <t>4c4cbe491f5e4c718e05f76ac5f35caa</t>
-  </si>
-  <si>
-    <t>4ce82c264f53486196ae07f5721275ba</t>
-  </si>
-  <si>
-    <t>4d0bf6ef7bc343b99948008d49bc8cc8</t>
-  </si>
-  <si>
-    <t>4d139cb82d314fd096c574e43d4c435d</t>
-  </si>
-  <si>
-    <t>4d606594acbe45a7899a0471dd91ccb0</t>
-  </si>
-  <si>
-    <t>4dae87cc1c6146b38dcbef082993c757</t>
-  </si>
-  <si>
-    <t>4e0dd03b43a74a99a0d243656ab34e91</t>
-  </si>
-  <si>
-    <t>4e62647f409447c59d7650eaa073f566</t>
-  </si>
-  <si>
-    <t>4e79c89726984936b3d1cf9392f2611f</t>
-  </si>
-  <si>
-    <t>4f38480c91ab4a5b8aab0943e43c1229</t>
-  </si>
-  <si>
-    <t>4f7e7c4216044d089b564a84457c6c98</t>
-  </si>
-  <si>
-    <t>4f9ad88381504ed4b7b3c64aa9db8225</t>
-  </si>
-  <si>
-    <t>4fb04772733d4d2885f603de292c2747</t>
-  </si>
-  <si>
-    <t>4fb36755336d442cbbcaf5905c5ba5b7</t>
-  </si>
-  <si>
-    <t>4fdbcdacebcc42dcb6e2e4d921fd03d7</t>
-  </si>
-  <si>
-    <t>500c4eb2c7114bac83de2ebab80f19bf</t>
-  </si>
-  <si>
-    <t>503942e6dcdf47299cbdc68f5bbb8df9</t>
-  </si>
-  <si>
-    <t>508644968c414d6ea0b5a917c297a5dc</t>
-  </si>
-  <si>
-    <t>5098d5d32b5842c89ae754cf7bb83f43</t>
-  </si>
-  <si>
-    <t>51050b87d8b248099d16bd60ca334b85</t>
-  </si>
-  <si>
-    <t>519fb08f36464d76ace65ced5548d020</t>
-  </si>
-  <si>
-    <t>51ae25dafefe45c28e48898b12e14a27</t>
-  </si>
-  <si>
-    <t>51d85b6fc5c04a1e8598857d19859c1e</t>
-  </si>
-  <si>
-    <t>5270502b270042e98965cebadedef1c9</t>
-  </si>
-  <si>
-    <t>529660e39a664f90a40cdc56714a8986</t>
-  </si>
-  <si>
-    <t>5299e2baa6964c4b910eb9f02b6f3cad</t>
-  </si>
-  <si>
-    <t>52da4da4176e4060b346ce8c426d2fff</t>
-  </si>
-  <si>
-    <t>52dad715b4084695b101591957014269</t>
-  </si>
-  <si>
-    <t>533946d5aa754b9a9fd909fba46ccebd</t>
-  </si>
-  <si>
-    <t>5340cffafc8f48439113e243d3e2ba28</t>
-  </si>
-  <si>
-    <t>5352591d82084d5fb25ddca4796b9805</t>
-  </si>
-  <si>
-    <t>540dc8d51784411893cd2d9319473fff</t>
-  </si>
-  <si>
-    <t>54114ffc770544b683528fcf4db81ed0</t>
-  </si>
-  <si>
-    <t>5419f1474cc44ad7b2bf58236238083f</t>
-  </si>
-  <si>
-    <t>5432c363bd824f6da24189280fe12e23</t>
-  </si>
-  <si>
-    <t>544f1e009492479e8f7230bee867a759</t>
-  </si>
-  <si>
-    <t>5466d9dd366140aa80dda524b31e709a</t>
-  </si>
-  <si>
-    <t>546a280c00514bc59a0a44cf38291c18</t>
-  </si>
-  <si>
-    <t>551cd2f0115d44188afbd1f89600bf9f</t>
-  </si>
-  <si>
-    <t>55eef18140724fc8889dffa68c599975</t>
-  </si>
-  <si>
-    <t>56c9291d97e84e69a62ac9d18a2a7252</t>
-  </si>
-  <si>
-    <t>5705096e40424bbe8bff95ed7e7d2adb</t>
-  </si>
-  <si>
-    <t>57a5bdfb4aca45178c4fd2659c4e1cfa</t>
-  </si>
-  <si>
-    <t>57dde08c5a8a4c2789bf6ba9d644f27b</t>
-  </si>
-  <si>
-    <t>581df5917fbb4c299531601787a9f447</t>
-  </si>
-  <si>
-    <t>58c566a54927438c8c24232cd7a1301c</t>
-  </si>
-  <si>
-    <t>58f67c485da141e99398fe90c4f64d00</t>
-  </si>
-  <si>
-    <t>590e95164ed64409b2b29ccc61cf476b</t>
-  </si>
-  <si>
-    <t>5971c366979948c3a5d776e7cb1446e6</t>
-  </si>
-  <si>
-    <t>5971c98b63c544edaef79f15e5919df4</t>
-  </si>
-  <si>
-    <t>5abe4d83bfe34526b9f69e69ecca40e0</t>
-  </si>
-  <si>
-    <t>5b63b900267840539f0ab23d5a08501d</t>
-  </si>
-  <si>
-    <t>5ba2d705f7704933b6ffeaff4c90c676</t>
-  </si>
-  <si>
-    <t>5ca391f9d144407d82ff544cbe402947</t>
-  </si>
-  <si>
-    <t>5cf36af5ef014e24a0a97f39d63159e2</t>
-  </si>
-  <si>
-    <t>5d7a36e3af25488faf4e6f4a295765ec</t>
-  </si>
-  <si>
-    <t>5d7f29f2736140feb64ca74527df51e5</t>
-  </si>
-  <si>
-    <t>5d8791bd7e74439aadb84277dbe948d9</t>
-  </si>
-  <si>
-    <t>5dc7d99d59244f23aa0152b58b6b98f4</t>
-  </si>
-  <si>
-    <t>5de29bae721045a98cbe326c62ebf246</t>
-  </si>
-  <si>
-    <t>5e28131be9074b838b83d3bb7ad2759c</t>
-  </si>
-  <si>
-    <t>5eb4a316da8f49d291fc34719539a8e4</t>
-  </si>
-  <si>
-    <t>5f9240e44de4452786d5e260606a4948</t>
-  </si>
-  <si>
-    <t>603597dea0e84591b2333d58e30835d6</t>
-  </si>
-  <si>
-    <t>605925a2736b4314b2b5b23bd52a838b</t>
-  </si>
-  <si>
-    <t>60b7ab3dc9b1420fb61fdc04ffae32f3</t>
-  </si>
-  <si>
-    <t>60e53ab8bfb0426ab323cb2a6be7c34a</t>
-  </si>
-  <si>
-    <t>60fcdf0e9c134309843d2ab9bc660cc9</t>
-  </si>
-  <si>
-    <t>613382d08bce4771bf306d0f97eca1d4</t>
-  </si>
-  <si>
-    <t>61e5032abeae4628b10a63986eb03624</t>
-  </si>
-  <si>
-    <t>628826321c494697ba962924606453d9</t>
-  </si>
-  <si>
-    <t>62ac5c757c98415fb2b7d259a164d4c7</t>
-  </si>
-  <si>
-    <t>62d4c3535e7a4d7bbbda3ecc17eb29ee</t>
-  </si>
-  <si>
-    <t>62e35054e4b646648be48909ff613153</t>
-  </si>
-  <si>
-    <t>63432f899e00472996b962be53f5de10</t>
-  </si>
-  <si>
-    <t>639d8b19a3ad4e789f12bcd5267046e7</t>
-  </si>
-  <si>
-    <t>63dd87154fd746f286e92b77b07ad49c</t>
-  </si>
-  <si>
-    <t>64407274a652406896afe546df5c47d1</t>
-  </si>
-  <si>
-    <t>64a3b71bff0648638246e93df7f5e253</t>
-  </si>
-  <si>
-    <t>64e0c1dd450549a09983e50713438620</t>
-  </si>
-  <si>
-    <t>64f5310b6e4941dd881060f7dc5cbc83</t>
-  </si>
-  <si>
-    <t>6549f309e161477286bdcddb9d512089</t>
-  </si>
-  <si>
-    <t>6598869deffa4040838f9c5e7ee27e2d</t>
-  </si>
-  <si>
-    <t>67452e22103d48bfb5b798ce8e0e2206</t>
-  </si>
-  <si>
-    <t>676b0c454782452b953f8ccf8360a64e</t>
-  </si>
-  <si>
-    <t>67dd97920952411e925fa7639730a490</t>
-  </si>
-  <si>
-    <t>67e05c4f47d6467da8e3dd28b3b4c884</t>
-  </si>
-  <si>
-    <t>68266ed11b0e4f1cb39dba8ebb82c187</t>
-  </si>
-  <si>
-    <t>68794b84db224c45a115f57a486a58a0</t>
-  </si>
-  <si>
-    <t>6889b84cd5684758ba9ad4cb7fda7d60</t>
-  </si>
-  <si>
-    <t>689c256e9bfb428e87721616ed71dd76</t>
-  </si>
-  <si>
-    <t>6951bab5bf3c4201961fc79fd19a324d</t>
-  </si>
-  <si>
-    <t>69e530e07ca0473e9a9b1c204f7ce649</t>
-  </si>
-  <si>
-    <t>6a582a6dc1e54ec3b08e7937ed4c5adc</t>
-  </si>
-  <si>
-    <t>6a5a59b80fbd4b3e945ee1ab3f4fd386</t>
-  </si>
-  <si>
-    <t>6a6eeb0a5a1b4d78bacf4477d6d17905</t>
-  </si>
-  <si>
-    <t>6a967dc1155d40be9c309cef658ffe4a</t>
-  </si>
-  <si>
-    <t>6ba5bdc839504099913d76e9697f74f6</t>
-  </si>
-  <si>
-    <t>6bf838a2fe8b4849a45b39c6e1e4c324</t>
-  </si>
-  <si>
-    <t>6c33c6ea219b473ba94147294eb3d2ba</t>
-  </si>
-  <si>
-    <t>6c413f2533f640819ec49b2c43c11eec</t>
-  </si>
-  <si>
-    <t>6c88f4ef03ab4cae84da3e8237b8251c</t>
-  </si>
-  <si>
-    <t>6ca5bbfdc8f74ab3a9f9bc87e749f163</t>
-  </si>
-  <si>
-    <t>6cad4354d22f4298b308847a3e36de6e</t>
-  </si>
-  <si>
-    <t>6cbeb40e518147e6848100a600da75cc</t>
-  </si>
-  <si>
-    <t>6cd1de92ef734b8c9367243e73de7d72</t>
-  </si>
-  <si>
-    <t>6ce964d13e8245578f72d22302d6e409</t>
-  </si>
-  <si>
-    <t>6d0593af719b468c9044e7a4b6ab2c75</t>
-  </si>
-  <si>
-    <t>6d0a7a1ffea84f04a123e1080253be15</t>
-  </si>
-  <si>
-    <t>6dbb5cdf8c49452bbf25c02b76f633fa</t>
-  </si>
-  <si>
-    <t>6dc1dbf66ee14c67921f717a0e3e933e</t>
-  </si>
-  <si>
-    <t>6e5575f50de44a1fb76732fe9b0d0aee</t>
-  </si>
-  <si>
-    <t>6ebab5e413e247059e4a628a7c246088</t>
-  </si>
-  <si>
-    <t>6f059c5266f641199846e0168fc4a3a7</t>
-  </si>
-  <si>
-    <t>6fb2a6bd66fe44b082f3d45c923a4dc0</t>
-  </si>
-  <si>
-    <t>7064cfc24aee4b5b9a0c50a7ebccfa8c</t>
-  </si>
-  <si>
-    <t>70a36077542b48fdb03b1d8dff3ffe67</t>
-  </si>
-  <si>
-    <t>70d762b518d846a7932565acd95b581e</t>
-  </si>
-  <si>
-    <t>7125f5426d384ccc99cade930805924b</t>
-  </si>
-  <si>
-    <t>71287fc9571c4ddd9e924764820fdf90</t>
-  </si>
-  <si>
-    <t>7216972f5ad24371b7b994945b62408e</t>
-  </si>
-  <si>
-    <t>730bfdbdacea4ae58e6e444a83fd5903</t>
-  </si>
-  <si>
-    <t>741fefafd7f34e64b9940c67c1135da1</t>
-  </si>
-  <si>
-    <t>74c7a0f17c274cc58d6d37bba5054ece</t>
-  </si>
-  <si>
-    <t>74efe0f068d84579bf8e996bb2cd5ce1</t>
-  </si>
-  <si>
-    <t>751c4dcaa3924301a7cd4d69bb3ef11d</t>
-  </si>
-  <si>
-    <t>75dcaefcd05e41d0b608440fcac1c00d</t>
-  </si>
-  <si>
-    <t>763d6d51ce29479da4f2b7086a7bc1b9</t>
-  </si>
-  <si>
-    <t>76caa14de4a44a49b6b2778d7a437cc9</t>
-  </si>
-  <si>
-    <t>76fc9cd4e8fa489ca616e81eccb6509b</t>
-  </si>
-  <si>
-    <t>76feb9cebde04b1faf8549dad2548673</t>
-  </si>
-  <si>
-    <t>7729f58533dc431b8e1464ef6e4f4c57</t>
-  </si>
-  <si>
-    <t>772f1174fe53442da3639e0b40ee9ce3</t>
-  </si>
-  <si>
-    <t>7780d0c9e80b4cbd8daaf0fb7f0cf9d7</t>
-  </si>
-  <si>
-    <t>77f805dafc804988a55659615f9ca454</t>
-  </si>
-  <si>
-    <t>78852ae947a14b83a7ecb0f770a7b096</t>
-  </si>
-  <si>
-    <t>78f6bf2b762849ff96ce9afd40490858</t>
-  </si>
-  <si>
-    <t>79172a72d3904499bc0abf77c76776b5</t>
-  </si>
-  <si>
-    <t>791ad042f6d7484581ffe3685cb375b7</t>
-  </si>
-  <si>
-    <t>7992d45b24ae436483f94471ea194af0</t>
-  </si>
-  <si>
-    <t>799346c6906a47a9bf8b2c341c337215</t>
-  </si>
-  <si>
-    <t>7a1ab0f3b2b7438bab060ac423556f20</t>
-  </si>
-  <si>
-    <t>7a3bc1c1eaee46668230413ee4ca5f4d</t>
-  </si>
-  <si>
-    <t>7a64b8cec1734033915de61df22b4351</t>
-  </si>
-  <si>
-    <t>7a98a251bd644c81b986c8ac7595ea02</t>
-  </si>
-  <si>
-    <t>7acac0d433584337930eca8e2c97f042</t>
-  </si>
-  <si>
-    <t>7b33e11c94d84fc688c6df2ef71cdb25</t>
-  </si>
-  <si>
-    <t>7b8dbd1bfed44cdb90b0e99451b545d2</t>
-  </si>
-  <si>
-    <t>7bf1161757814db3b3139c29f930cec7</t>
-  </si>
-  <si>
-    <t>7c101d72bef942e88665cd0788b2558e</t>
-  </si>
-  <si>
-    <t>7c4c8c7ac4754fe3a92f178feb944c2a</t>
-  </si>
-  <si>
-    <t>7c9fe018c92b47ce8f805707388198a8</t>
-  </si>
-  <si>
-    <t>7d7f567e5b96447c8fb1db327b503967</t>
-  </si>
-  <si>
-    <t>7da053bc84f04902a40d3d20b2e13a84</t>
-  </si>
-  <si>
-    <t>7e364f411d91408293327bff7288876e</t>
-  </si>
-  <si>
-    <t>7f93801289af41e4a07bb2c9f7c2a1a5</t>
-  </si>
-  <si>
-    <t>7fc347bfdbab4ff28c1e774266ed8b24</t>
-  </si>
-  <si>
-    <t>8045b510fe174e5fb8ee64966d90f4a7</t>
-  </si>
-  <si>
-    <t>8053f0a2bf3a4666831756531ef708de</t>
-  </si>
-  <si>
-    <t>807da4ea7e6d4cb1b0f29d06741d7dc6</t>
-  </si>
-  <si>
-    <t>809805f0c662499d99618e98c7e8104f</t>
-  </si>
-  <si>
-    <t>80a111ccd3c04acea69711dceb3571a5</t>
-  </si>
-  <si>
-    <t>80f9c3683ed0403892d83d389c278930</t>
-  </si>
-  <si>
-    <t>8115ebb22a0548a79f641909510fbd68</t>
-  </si>
-  <si>
-    <t>815ccc5bb4a64b2896f1438bd720c178</t>
-  </si>
-  <si>
-    <t>8197a619acf54ba98bf34d7b8b00855f</t>
-  </si>
-  <si>
-    <t>8219cc0338294de9bed0cc5bc1395d35</t>
-  </si>
-  <si>
-    <t>821ea306dada42d9bbffa47eea5026f4</t>
-  </si>
-  <si>
-    <t>823c0ac247534a07a3a055f8f48598c8</t>
-  </si>
-  <si>
-    <t>8245b4e6e83740218b6ba451f94584b5</t>
-  </si>
-  <si>
-    <t>829d016255d04902bb71e1464bd2f3b2</t>
-  </si>
-  <si>
-    <t>82fd87575f774ed9b9a86c75efb2efa5</t>
-  </si>
-  <si>
-    <t>82febff30d0b4fc88c781c8c4c9f3ed6</t>
-  </si>
-  <si>
-    <t>8304db00749e46fc879e1f0f9e0c42ad</t>
-  </si>
-  <si>
-    <t>8322c38a7b5b4cdb9c4164ff752d2157</t>
-  </si>
-  <si>
-    <t>8338bc064ac1493da5b1678938e295b5</t>
-  </si>
-  <si>
-    <t>83434c05384d4901b3875602b66d5860</t>
-  </si>
-  <si>
-    <t>83a3deda5e3b42b8957ffef3f27126de</t>
-  </si>
-  <si>
-    <t>83aa7dbb71b3435d8a5bba0bd47859ff</t>
-  </si>
-  <si>
-    <t>83ad11f5992d431a9186bdaee66deaad</t>
-  </si>
-  <si>
-    <t>841918cc247f4a1c9ae984aff0cda083</t>
-  </si>
-  <si>
-    <t>8456a02add3342afb3c5ae5fa5d2f3c4</t>
-  </si>
-  <si>
-    <t>8578d331d25d45a288ae730cda41baa6</t>
-  </si>
-  <si>
-    <t>858a69831b16424b83253791a551eb78</t>
-  </si>
-  <si>
-    <t>85fb226fa0944ebeb3b96eff220319da</t>
-  </si>
-  <si>
-    <t>8642e2e756c6450e806b1dd3d3e296cb</t>
-  </si>
-  <si>
-    <t>864eed5c80384a69a2c6aedf55f19be5</t>
-  </si>
-  <si>
-    <t>869130e87ae84894ac91805cc57a29d3</t>
-  </si>
-  <si>
-    <t>878cb5b7960a448d8f3604e7eacb4784</t>
-  </si>
-  <si>
-    <t>883a6456dea24dcf8a50dd64ebc0f90e</t>
-  </si>
-  <si>
-    <t>885532ca14b74d3fb4ba0c100ae3613a</t>
-  </si>
-  <si>
-    <t>8891645dbcdb4865aa53ccd2e574db4f</t>
-  </si>
-  <si>
-    <t>889fa5c5027b4ef4ba2f311b41200400</t>
-  </si>
-  <si>
-    <t>88a4c240ef04452990bd3b230508240f</t>
-  </si>
-  <si>
-    <t>89251dea945d4dcc98c314b4084a630e</t>
-  </si>
-  <si>
-    <t>8938ebcb79dc419cb779e3ecfb82e6bd</t>
-  </si>
-  <si>
-    <t>895cb58537294c4287885bf38f5841d0</t>
-  </si>
-  <si>
-    <t>898b862b47554b6ba3321f45dcb86bc5</t>
-  </si>
-  <si>
-    <t>89e23802101c4793887ddaa73b665d09</t>
-  </si>
-  <si>
-    <t>8a7e8ee004244872ac1bbb939f0c7405</t>
-  </si>
-  <si>
-    <t>8b38841766124c16a4024a8dc5047cdd</t>
-  </si>
-  <si>
-    <t>8b5d1bcc6fda419fbae1cd5aa5273f7b</t>
-  </si>
-  <si>
-    <t>8b8728a2392b4c6e9fd36959b2977003</t>
-  </si>
-  <si>
-    <t>8bbe7dbfbf404aaeb71ea4b7672ff037</t>
-  </si>
-  <si>
-    <t>8bc31023753e455a883a5782096b5730</t>
-  </si>
-  <si>
-    <t>8bf7ace8d6174693944bcd15ce4dd813</t>
-  </si>
-  <si>
-    <t>8d048f2fa7c44e928e36805d54d9dd8a</t>
-  </si>
-  <si>
-    <t>8d70b2b1973b4e78b7481bae68758f06</t>
-  </si>
-  <si>
-    <t>8d8492306155451b934e7eee39b7ff0a</t>
-  </si>
-  <si>
-    <t>8d9120ab09c541e9bc55c3a83e36923d</t>
-  </si>
-  <si>
-    <t>8e3acbc7ef7a4c21b4f369e75c173e9c</t>
-  </si>
-  <si>
-    <t>8e502af9f25b4173b1e8462d8371b77f</t>
-  </si>
-  <si>
-    <t>8e928ead7de647c188296ae9c996ffbd</t>
-  </si>
-  <si>
-    <t>8ef352567cdc4308bcca155b5b5fac8d</t>
-  </si>
-  <si>
-    <t>8f317fbe1b5446a4bb595af6a3c63555</t>
-  </si>
-  <si>
-    <t>8f4cd5f09cf744099318e6b97b6dd388</t>
-  </si>
-  <si>
-    <t>8ffda1695d554a809bc10f0c90de28d5</t>
-  </si>
-  <si>
-    <t>90bc976337ee424886ec88811fbdd02d</t>
-  </si>
-  <si>
-    <t>90d6220a1d3e412ea3371af55afe2840</t>
-  </si>
-  <si>
-    <t>90da8b3f568d44c09d6e3f80df3bd8e5</t>
-  </si>
-  <si>
-    <t>918aa17f84154910b46f44b05af9c61a</t>
-  </si>
-  <si>
-    <t>91feb7fe0c4b42328bebca9df70cd099</t>
-  </si>
-  <si>
-    <t>925346e61c3445fb831c035bbfacd08d</t>
-  </si>
-  <si>
-    <t>9274f98bb3b84229b4250aac875562fb</t>
-  </si>
-  <si>
-    <t>92cff302087646bd900420524f222287</t>
-  </si>
-  <si>
-    <t>931ab287445a482897c922b1302cb144</t>
-  </si>
-  <si>
-    <t>93770ead7e3a43ddb676af76651eda75</t>
-  </si>
-  <si>
-    <t>948260ec97b44fcfa5ebb47fd18c9ba4</t>
-  </si>
-  <si>
-    <t>94c298d0772d42189ed250cc4691616b</t>
-  </si>
-  <si>
-    <t>95000fc8e3384056abfd17d3b7bb25f3</t>
-  </si>
-  <si>
-    <t>950960fd052849e0ab46c2f26c853a98</t>
-  </si>
-  <si>
-    <t>9552899ee96b43688276ebc54ab3d92a</t>
-  </si>
-  <si>
-    <t>960b604e6d4346c5b9107b3b68f92088</t>
-  </si>
-  <si>
-    <t>96104e72d7124f3caaaa389cd9881fe4</t>
-  </si>
-  <si>
-    <t>969264a324ce4a2fa07395923337ed41</t>
-  </si>
-  <si>
-    <t>96b926b5d6364608b06163e3a752cdcd</t>
-  </si>
-  <si>
-    <t>96bc83b60a78463294adbfa3b5e9839e</t>
-  </si>
-  <si>
-    <t>96c26c47dc4640c4880a57286c0e7989</t>
-  </si>
-  <si>
-    <t>96d2ca190e614ff48e7d904b8538412d</t>
-  </si>
-  <si>
-    <t>975c0d44804d455d80e087fba9cf3f35</t>
-  </si>
-  <si>
-    <t>979d3086ce25422da8a91e89adf19ab7</t>
-  </si>
-  <si>
-    <t>97e47ee727ac48c4a18dd1c5b911800f</t>
-  </si>
-  <si>
-    <t>97f20073257d41a1ad1d0bd562805a17</t>
-  </si>
-  <si>
-    <t>98bbb475d7f74bec9246103616dfb619</t>
-  </si>
-  <si>
-    <t>99361b798a85406ab66fdeb6ff78a07e</t>
-  </si>
-  <si>
-    <t>99bf4ecb7b9448129dfda06b063a1394</t>
-  </si>
-  <si>
-    <t>99bf8fec004c410d9de5dc57c66f6218</t>
-  </si>
-  <si>
-    <t>99e48acff13e4b2e8bdfcde51e44f99f</t>
-  </si>
-  <si>
-    <t>9a1ce6e572194ed293ba04e926d2a356</t>
-  </si>
-  <si>
-    <t>9a86c9cf8a1947bda0ec80d4c69d4ccf</t>
-  </si>
-  <si>
-    <t>9ac974702a6b4fa99cbaaf182775b381</t>
-  </si>
-  <si>
-    <t>9b0cf0b9277b467984f8716dd7f3b564</t>
-  </si>
-  <si>
-    <t>9b31977b210640a9a73cee23b6956daf</t>
-  </si>
-  <si>
-    <t>9be84cfa12864667aa51e2d7e0c668c6</t>
-  </si>
-  <si>
-    <t>9c368b702a1e4e88b35d0ff2395d3b5e</t>
-  </si>
-  <si>
-    <t>9c8a8ee2efc54160b3a239f66da9403b</t>
-  </si>
-  <si>
-    <t>9ca2b8167d4647f492f4b92b463e873e</t>
-  </si>
-  <si>
-    <t>9cad292c6f8f423eab95f12cd8da11e1</t>
-  </si>
-  <si>
-    <t>9cfb01c01d1645e78284b81a2d849350</t>
-  </si>
-  <si>
-    <t>9d84b0ff1c46461faeafafd26645bc1d</t>
-  </si>
-  <si>
-    <t>9db3163fe12e41b2a66368007bc50f8c</t>
-  </si>
-  <si>
-    <t>9e481656b9014fda85629b4753ae6eb7</t>
-  </si>
-  <si>
-    <t>9e94ac5efa4448ae82ccb3abfcf9e5b8</t>
-  </si>
-  <si>
-    <t>9ed73aa136f54131a4fa097e08e3ced3</t>
-  </si>
-  <si>
-    <t>9ee14c6aad854dbfb7d0ccc055efcf27</t>
-  </si>
-  <si>
-    <t>9f15671d77c84f12bb99f2f6cb82ad2c</t>
-  </si>
-  <si>
-    <t>9f842b71cb9b4f5985f98d33ea0838a7</t>
-  </si>
-  <si>
-    <t>9fd58d1ae2784405bf18d57d710d1d6c</t>
-  </si>
-  <si>
-    <t>a07773571fc44680a9ade6c6313c6cb2</t>
-  </si>
-  <si>
-    <t>a081e11b611b41f5826c18985028aab3</t>
-  </si>
-  <si>
-    <t>a0a475f305db4a929357934d2184e029</t>
-  </si>
-  <si>
-    <t>a0aff05d58884a0ea880c6b30ee47c71</t>
-  </si>
-  <si>
-    <t>a0b5601a51794171813cc60c634a3a12</t>
-  </si>
-  <si>
-    <t>a0dcb55b148045c4b2da226bfbe87f68</t>
-  </si>
-  <si>
-    <t>a0e85e26b67e46b6a0d1df64d21fd20c</t>
-  </si>
-  <si>
-    <t>a1c94b20badd45e0ac99eacdc68cc4a1</t>
-  </si>
-  <si>
-    <t>a210fbb4a0bf4edeab19b0c5361fe981</t>
-  </si>
-  <si>
-    <t>a22ea790bdfa409fb0ea5396a4c8e689</t>
-  </si>
-  <si>
-    <t>a24b6edfd5144d168ef2359fa104dd0c</t>
-  </si>
-  <si>
-    <t>a2694e26387f4d61af76e4f29d68cc0f</t>
-  </si>
-  <si>
-    <t>a2c7d846fc2746b29e1785eb5f95ae67</t>
-  </si>
-  <si>
-    <t>a37e069323ac48128da83ec49a7a4914</t>
-  </si>
-  <si>
-    <t>a448ae49c6dc44a78c22e039793692d4</t>
-  </si>
-  <si>
-    <t>a48cdea4e4f048788a5e27eadf3be278</t>
-  </si>
-  <si>
-    <t>a4e93094820f403184fda3795acd39f7</t>
-  </si>
-  <si>
-    <t>a4fa03bd576746bc90de7ee835368786</t>
-  </si>
-  <si>
-    <t>a59e6291369645e39eaed1f7be75b711</t>
-  </si>
-  <si>
-    <t>a67df296e4014a82a3d9382f5c6c35a4</t>
-  </si>
-  <si>
-    <t>a6a12698ed814565a92965d2aeb8638e</t>
-  </si>
-  <si>
-    <t>a6cc1e367c944155b346d6f5a1af18e4</t>
-  </si>
-  <si>
-    <t>a73c01db93b24c38969d02ce55b27ac4</t>
-  </si>
-  <si>
-    <t>a73e7fb9ced345c4829275e087b658da</t>
-  </si>
-  <si>
-    <t>a75418df2db442978c43cda055fac5f4</t>
-  </si>
-  <si>
-    <t>a7673f6391de4e2da8f1be68407bd729</t>
-  </si>
-  <si>
-    <t>a81c21aeb11745b598154c362a579e85</t>
-  </si>
-  <si>
-    <t>a8599af66eab4ae0ae4f771f7b164533</t>
-  </si>
-  <si>
-    <t>a8ae6b66f81f4aeb82d081502629690a</t>
-  </si>
-  <si>
-    <t>a9f683786c7a46e7942e14aaa6de3069</t>
-  </si>
-  <si>
-    <t>aa419dfe3e10431d98fb09e9cdeee359</t>
-  </si>
-  <si>
-    <t>ab1d885df1f4497b87b9d6bd5b56a488</t>
-  </si>
-  <si>
-    <t>aba63765058e4929b70027c7d8ed259e</t>
-  </si>
-  <si>
-    <t>abc08c614a794c589c083073daeba469</t>
-  </si>
-  <si>
-    <t>abf0c106c397450987e43aaad020f313</t>
-  </si>
-  <si>
-    <t>ac349cc771cb42739284c14b4bb27099</t>
-  </si>
-  <si>
-    <t>ac534a22fd0b440fb17d42b8a042a5c1</t>
-  </si>
-  <si>
-    <t>ac561416e52847d68af3c46cadd4c34c</t>
-  </si>
-  <si>
-    <t>ac7b9d4328e8425bb5a13aeac3d3946a</t>
-  </si>
-  <si>
-    <t>acbb6a35b6bc40eea6da594d025234e5</t>
-  </si>
-  <si>
-    <t>acc7d59e7b8b4a8bb28d327127a06e62</t>
-  </si>
-  <si>
-    <t>acef8ca97ced456db520d9ee5d551870</t>
-  </si>
-  <si>
-    <t>ad2cc9554ac242c8b4c01c724c72aa9f</t>
-  </si>
-  <si>
-    <t>ad721105c9644a3f8d3c682f896eaadd</t>
-  </si>
-  <si>
-    <t>ad947ee4689e4f58a933aed06196943b</t>
-  </si>
-  <si>
-    <t>ae23c85270764529a6346a5c04d8b17f</t>
-  </si>
-  <si>
-    <t>ae5574744c35411291df4147bfde363f</t>
-  </si>
-  <si>
-    <t>ae66d16850c744d9aa2feb638d5b7a63</t>
-  </si>
-  <si>
-    <t>ae7c64816cf94de591a5a2ac4c1ec7c3</t>
-  </si>
-  <si>
-    <t>aefa452b60004ac3a330b8357d6eaae4</t>
-  </si>
-  <si>
-    <t>aeff858b1c9c41629d4369bad966c3c7</t>
-  </si>
-  <si>
-    <t>af0a38c8905c4b228940919a66d4d39c</t>
-  </si>
-  <si>
-    <t>af33d5111357436b8e80d7898642295b</t>
-  </si>
-  <si>
-    <t>af476b609d9746d3ac3e56dcc98faa0b</t>
-  </si>
-  <si>
-    <t>af81f4aa3e68445a85d6c260ecb16bf3</t>
-  </si>
-  <si>
-    <t>af8a48750d4a417f9dbfbe0930e939e1</t>
-  </si>
-  <si>
-    <t>aff354b8212640ff94998a71493e9b43</t>
-  </si>
-  <si>
-    <t>b007292a216147b0892c0084657a8436</t>
-  </si>
-  <si>
-    <t>b0386e46e0064a71b21f63f2455c6200</t>
-  </si>
-  <si>
-    <t>b0b3666b855947b781fb1e8fa4de1c0b</t>
-  </si>
-  <si>
-    <t>b0b8e348aebf4a6d966d92e547e3859f</t>
-  </si>
-  <si>
-    <t>b1e16b89992445aa9ff431afbceedd1e</t>
-  </si>
-  <si>
-    <t>b212ed0876014fd09824661f485c4388</t>
-  </si>
-  <si>
-    <t>b25fa3b44ab241e4bd0ee70f387a1deb</t>
-  </si>
-  <si>
-    <t>b283a0e5808447f991ef9840f1ecc076</t>
-  </si>
-  <si>
-    <t>b2de7a1eab7f4c5580388c8d640fba31</t>
-  </si>
-  <si>
-    <t>b2f769cd3cbf4693a86d35561fead070</t>
-  </si>
-  <si>
-    <t>b318d5f1baba479b989473a8b61ed6c3</t>
-  </si>
-  <si>
-    <t>b3b5b9a680cc4e289ba989ca6e45f02b</t>
-  </si>
-  <si>
-    <t>b3d9a424cdd64078911421b1d633b8bf</t>
-  </si>
-  <si>
-    <t>b3e4df36f2af48c68d65de1e4d6c62c4</t>
-  </si>
-  <si>
-    <t>b4292728cbb84e0591d5486c2cbfe6be</t>
-  </si>
-  <si>
-    <t>b44ab99283e549ffbd43c65f95a2a33c</t>
-  </si>
-  <si>
-    <t>b4b6d86a1ece4a9ea29314454496484a</t>
-  </si>
-  <si>
-    <t>b4d7b91ca4164c99ade94230af639f4e</t>
-  </si>
-  <si>
-    <t>b5762c5fcfce4fd794093d7d4ca45b73</t>
-  </si>
-  <si>
-    <t>b697eb9219424e0ba34e603f3b26920b</t>
-  </si>
-  <si>
-    <t>b6ca6915981d4bde8fe52e0c8a596c85</t>
-  </si>
-  <si>
-    <t>b6ffdf92784a41e9a3087a4e5f2d0e41</t>
-  </si>
-  <si>
-    <t>b71e193570ec41b9a78f559596039209</t>
-  </si>
-  <si>
-    <t>b78500fe0e344ef29e6f1b4702f0da22</t>
-  </si>
-  <si>
-    <t>b78a3ebc17bb4fc9bbacaf13f2b863ea</t>
-  </si>
-  <si>
-    <t>b7fd426db2734ce8b4fdee555d65dd67</t>
-  </si>
-  <si>
-    <t>b8321499d19f4396b3cb7473d6c98e38</t>
-  </si>
-  <si>
-    <t>b8951dcdd82e44d0863d3e1af1f46240</t>
-  </si>
-  <si>
-    <t>b8a1bea44a484c108a7c14ff6269c474</t>
-  </si>
-  <si>
-    <t>b8a5fd80d43c4a088095ab31e8ad3245</t>
-  </si>
-  <si>
-    <t>b9873f9cdfbf43488e68982ae84d7d02</t>
-  </si>
-  <si>
-    <t>b9e8726e28de49499432981799a2148a</t>
-  </si>
-  <si>
-    <t>ba56efc6cb184eb6a587ac0b99bb7965</t>
-  </si>
-  <si>
-    <t>bb1f939a58104070ad7cbb71208281b2</t>
-  </si>
-  <si>
-    <t>bb5866d2744f4d84a9be0d79dbd00806</t>
-  </si>
-  <si>
-    <t>bbce1abf05754b28a12875169c85857d</t>
-  </si>
-  <si>
-    <t>bc1151cfbb8f4d9fb70ba4a3548358da</t>
-  </si>
-  <si>
-    <t>bc1c843858174f80af5a850cf2d2a47e</t>
-  </si>
-  <si>
-    <t>bc69772de2a540f0821fe9ccb7be914d</t>
-  </si>
-  <si>
-    <t>bc89282f70b449238731dee10a93c26d</t>
-  </si>
-  <si>
-    <t>bd955aed86fd43e4acc21484521c461f</t>
-  </si>
-  <si>
-    <t>bdae21677d9849a699b5f04fb9794dfa</t>
-  </si>
-  <si>
-    <t>bdec04f24f8c496db09b4c48601b432b</t>
-  </si>
-  <si>
-    <t>be1668fa727848899fc6a6c89b62a903</t>
-  </si>
-  <si>
-    <t>be45b80eb7da4b38998f9a0f767d4a2b</t>
-  </si>
-  <si>
-    <t>bf3976f951d74f1298189f9b1a7c5981</t>
-  </si>
-  <si>
-    <t>bf7ee9d5cca74f8ea3561b8a4c7b1fb2</t>
-  </si>
-  <si>
-    <t>bf8fed70d27f431cb65d8858b8a283c4</t>
-  </si>
-  <si>
-    <t>bfb9a662b58c482fa2534fb5d5b8f56d</t>
-  </si>
-  <si>
-    <t>c07b81dd7efc40ac8b5037aa706548fd</t>
-  </si>
-  <si>
-    <t>c07e69db9afc455ba2c1b4b5654c9edf</t>
-  </si>
-  <si>
-    <t>c0826e4ee5e34228a6f5779f19ad182a</t>
-  </si>
-  <si>
-    <t>c0f9984821db4e38baf4b2d4e62a180c</t>
-  </si>
-  <si>
-    <t>c1215fc0199f40c3adeeb190a9990731</t>
-  </si>
-  <si>
-    <t>c1ac7445a07e431ebefc5471278d083d</t>
-  </si>
-  <si>
-    <t>c2140644e7a24d668095c058296fa29b</t>
-  </si>
-  <si>
-    <t>c26f8d69f3504253bb09977bc3f666f7</t>
-  </si>
-  <si>
-    <t>c27125e822064c6690f98654fa9ec762</t>
-  </si>
-  <si>
-    <t>c342f4e1937a49839ec23caf171831df</t>
-  </si>
-  <si>
-    <t>c347c049d83f4eb794a0a8f3cabe4878</t>
-  </si>
-  <si>
-    <t>c4b4f712658c43bc91c163477a7e6422</t>
-  </si>
-  <si>
-    <t>c5254eecffe545b8934ec5a0d0327932</t>
-  </si>
-  <si>
-    <t>c57b7b04985f4a34b2c2e2b87a102e06</t>
-  </si>
-  <si>
-    <t>c581a65b42a44d94a145b71934cb0ee9</t>
-  </si>
-  <si>
-    <t>c5a792fff065465ea4883ecd296171a6</t>
-  </si>
-  <si>
-    <t>c5c24b91030848ca987c908aa8fd570f</t>
-  </si>
-  <si>
-    <t>c5f931f31e8d450281d49fed8a3a4836</t>
-  </si>
-  <si>
-    <t>c65f786eee5640cdbe9245d7f2efafbc</t>
-  </si>
-  <si>
-    <t>c7fa537fa92747049d9f4c80db955e10</t>
-  </si>
-  <si>
-    <t>c93aa9c4278a46a08711bbe9aa93e6cd</t>
-  </si>
-  <si>
-    <t>c9584d0672944d749356550e2a6ca42b</t>
-  </si>
-  <si>
-    <t>c97a7dd7e08542fe99ec5d74547cb2e7</t>
-  </si>
-  <si>
-    <t>c99e66b0bd2b4fd7865e345e62d2bb35</t>
-  </si>
-  <si>
-    <t>c9f18bf263b343a9a005c0f01f00c89d</t>
-  </si>
-  <si>
-    <t>ca112e2341a347b8b50eada57684b1e2</t>
-  </si>
-  <si>
-    <t>ca157284c8d34cacbd0d6b0b1f85cab1</t>
-  </si>
-  <si>
-    <t>ca2cdc48786f451dac29e80631264c61</t>
-  </si>
-  <si>
-    <t>ca8c01a3794e4c7b92fc5b53118c5efc</t>
-  </si>
-  <si>
-    <t>cb073907d406430a9e6d39bbbfcc22a6</t>
-  </si>
-  <si>
-    <t>cc1ceae1a69e4da0b7299f0d35bf09da</t>
-  </si>
-  <si>
-    <t>cc465c539efa4fa68db9799b8e399f78</t>
-  </si>
-  <si>
-    <t>cc9c27f85e294bdcb54c6677ef32bcbb</t>
-  </si>
-  <si>
-    <t>cc9e362b3af94f809d9d6f1ec385569c</t>
-  </si>
-  <si>
-    <t>ccaca507fa9b4e98ba63e476cdb32068</t>
-  </si>
-  <si>
-    <t>cd27630789974208af160a8f9426fb97</t>
-  </si>
-  <si>
-    <t>cd3ef41cf37b44a0a4a78867217d4bdc</t>
-  </si>
-  <si>
-    <t>cd4ed2da251b4b7eb7fd7961e5a378dd</t>
-  </si>
-  <si>
-    <t>cd574d5c770b4e8a87a8528b6826c9e1</t>
-  </si>
-  <si>
-    <t>cd5dff7079d5428eb50447e6e6e017f3</t>
-  </si>
-  <si>
-    <t>cd92d00932b14da5b111d50ecbbe6564</t>
-  </si>
-  <si>
-    <t>cdb3f421e3a44272aaa88250fdc9b4bd</t>
-  </si>
-  <si>
-    <t>cddc023cfd764a9b83066920d4cf5b3b</t>
-  </si>
-  <si>
-    <t>ce0577b9863a4f50906a43de693051eb</t>
-  </si>
-  <si>
-    <t>ce7c427063264c069df1c1ec9ad55ebf</t>
-  </si>
-  <si>
-    <t>cec919b262cf4c13a97249d20da14b12</t>
-  </si>
-  <si>
-    <t>cf9862ce0fe14915afb38db4117c8484</t>
-  </si>
-  <si>
-    <t>cfbcd0efdb8c4e99ae51d9b459b69e96</t>
-  </si>
-  <si>
-    <t>d000f090ebfb4bd683e2c00bbc5ecb28</t>
-  </si>
-  <si>
-    <t>d003ec4d773545eeabdcc6b8c84ae555</t>
-  </si>
-  <si>
-    <t>d02a38e5a7454066ad95094b808fbd3e</t>
-  </si>
-  <si>
-    <t>d03cabe5791f4226823282488fa65277</t>
-  </si>
-  <si>
-    <t>d0bfc5cab6744172a800e637e03ccad3</t>
-  </si>
-  <si>
-    <t>d107797fbe174b21a2ebfb8a8cb80168</t>
-  </si>
-  <si>
-    <t>d16dd4e795b946f180bbde0bd6d9532f</t>
-  </si>
-  <si>
-    <t>d1ce57145b144f0089127e29635d1c87</t>
-  </si>
-  <si>
-    <t>d22a1958e26446f0b50bd3cb5545761f</t>
-  </si>
-  <si>
-    <t>d25cbc486b3548d28494b6d57294ea63</t>
-  </si>
-  <si>
-    <t>d3747bc49a0e463c98364a826d75606f</t>
-  </si>
-  <si>
-    <t>d3945f7128fc45d1967194e929101620</t>
-  </si>
-  <si>
-    <t>d3ca36a764f044468ec7cd3aa31fa46a</t>
-  </si>
-  <si>
-    <t>d3d82d5e9f8340a786676336a937e2c0</t>
-  </si>
-  <si>
-    <t>d40ec9d2465c41638de6fafdc5915b97</t>
-  </si>
-  <si>
-    <t>d48884bbff464bfd9b3a0fea2423c7dc</t>
-  </si>
-  <si>
-    <t>d49485b9c2c74a09b2689037c39ad90f</t>
-  </si>
-  <si>
-    <t>d4ad867360c942f5bce8693fe5562ec7</t>
-  </si>
-  <si>
-    <t>d4bb9a51ad0f4f3e88e678c39f84437b</t>
-  </si>
-  <si>
-    <t>d4ff915e9efc41cb81c5309f9bda4c8e</t>
-  </si>
-  <si>
-    <t>d53ff72d7360469692cc3e0497ee9dde</t>
-  </si>
-  <si>
-    <t>d560fd567f1c4430926de354789816c9</t>
-  </si>
-  <si>
-    <t>d65031db5d9148cab82e340b437b3f3c</t>
-  </si>
-  <si>
-    <t>d6f4cf6fa7ed46f198cefd2e35bb9de3</t>
-  </si>
-  <si>
-    <t>d706d14373f84490a4006a3d75f76b1d</t>
-  </si>
-  <si>
-    <t>d8670f18bb64475ab58bac36473778d8</t>
-  </si>
-  <si>
-    <t>d87283528b994c66aabc927d8c105df2</t>
-  </si>
-  <si>
-    <t>d879ef9358cd4add96ffb75a8ed45766</t>
-  </si>
-  <si>
-    <t>d8c51de27096426db774b2bb210ecaf7</t>
-  </si>
-  <si>
-    <t>d8d5c98331fd44a49b61f1addc617171</t>
-  </si>
-  <si>
-    <t>d945c0d23e684504ae5e43b17bd8c217</t>
-  </si>
-  <si>
-    <t>daa556128e09439f973e5cbb59e2a1c6</t>
-  </si>
-  <si>
-    <t>dba2b01b919444ce8086e868f23cbeff</t>
-  </si>
-  <si>
-    <t>dbb7d49c82a34e9fa5ae37fcecd69980</t>
-  </si>
-  <si>
-    <t>dbed3628d65e4631896dd9be766d4bed</t>
-  </si>
-  <si>
-    <t>dc92eb0846a04cbbaf71c37da9fd669a</t>
-  </si>
-  <si>
-    <t>dd0861f96eed424b85afcfa8815e7e73</t>
-  </si>
-  <si>
-    <t>de841b5bde664c4d847341103007795c</t>
-  </si>
-  <si>
-    <t>df2425e36639489fa58fb3e6e9e97054</t>
-  </si>
-  <si>
-    <t>e03b181791b84d2f8d3e8845d5c331eb</t>
-  </si>
-  <si>
-    <t>e12ea0d6bf544dc98e0ad9c4c19378a1</t>
-  </si>
-  <si>
-    <t>e137c0923a624d2382484755dd4dedd6</t>
-  </si>
-  <si>
-    <t>e145f3b7200946c6bb27d1f8a289a34d</t>
-  </si>
-  <si>
-    <t>e15f6b97801d436bbc1c6443c2e3798d</t>
-  </si>
-  <si>
-    <t>e174cb26e8ef4c63a268877ef6920439</t>
-  </si>
-  <si>
-    <t>e1882176aa4842d98fc960df4f1a6fd3</t>
-  </si>
-  <si>
-    <t>e211bb56c246494fad621839575f2eb6</t>
-  </si>
-  <si>
-    <t>e24388cf071b4c40a7b72c7ce288d0c5</t>
-  </si>
-  <si>
-    <t>e245b8632d804a9fbad5aa55b3615f17</t>
-  </si>
-  <si>
-    <t>e2e9e05ac367436c93bb45744c875392</t>
-  </si>
-  <si>
-    <t>e3700dd6382d4dd09b1c5ff4d743a6b4</t>
-  </si>
-  <si>
-    <t>e381a72f4aea443aac259516575618aa</t>
-  </si>
-  <si>
-    <t>e397ce3633d6499c8cb8be8cc07b2b3c</t>
-  </si>
-  <si>
-    <t>e45d49c4df604d52973b5907fba8db5b</t>
-  </si>
-  <si>
-    <t>e4fe2a7856da4cdea533d353c5ebfe5f</t>
-  </si>
-  <si>
-    <t>e576368b1af24e5c9bca8f9b0409802b</t>
-  </si>
-  <si>
-    <t>e5e2df555a8f4b4195e03e446abffd34</t>
-  </si>
-  <si>
-    <t>e63e1315e2674fd6a9d5be6c43940dec</t>
-  </si>
-  <si>
-    <t>e69178acbdea41ed9bfc5c89cb280956</t>
-  </si>
-  <si>
-    <t>e6ee6b3ef526462d9c8ff64068883a28</t>
-  </si>
-  <si>
-    <t>e75b7d3eb7f14109a29c4635674ea1cf</t>
-  </si>
-  <si>
-    <t>e84adb233e66403fba8d1d1ebbc06db3</t>
-  </si>
-  <si>
-    <t>e8731ba292d34f809977cadc8344c10d</t>
-  </si>
-  <si>
-    <t>e8cea7e1fadf4e618e1d8237e172c381</t>
-  </si>
-  <si>
-    <t>e99974c88a53468abc7b2d545e9bade0</t>
-  </si>
-  <si>
-    <t>e9ba8d7deb5f451f98c2e3951131f4d6</t>
-  </si>
-  <si>
-    <t>e9f5d446f0964877b575043c3f70afec</t>
-  </si>
-  <si>
-    <t>ea2822b6ced24e13ba5627ed80038264</t>
-  </si>
-  <si>
-    <t>ea79172526a8479eaf1a2a80cb046294</t>
-  </si>
-  <si>
-    <t>ea9d68def8a3440ebfb4153d47e006b6</t>
-  </si>
-  <si>
-    <t>eb3357022cc84dbb95ff0574c5738eec</t>
-  </si>
-  <si>
-    <t>eb6541bf0b454a9ea53113c8bf27bf7a</t>
-  </si>
-  <si>
-    <t>eb77467c6ea24d4ca3e1112677e0b45a</t>
-  </si>
-  <si>
-    <t>ebc3ce530a6c42d6b7cdcd111fbc981c</t>
-  </si>
-  <si>
-    <t>ebd10bd148d74d58b7704d2cd88255f5</t>
-  </si>
-  <si>
-    <t>ebfc55b33b66415792b55224ec80f004</t>
-  </si>
-  <si>
-    <t>ec89260ebb99452c9a265f115f15fb83</t>
-  </si>
-  <si>
-    <t>ecf9d90cb66c435ba508b77c811134be</t>
-  </si>
-  <si>
-    <t>ed06a939546a4b5f9820d3d58488f3df</t>
-  </si>
-  <si>
-    <t>ed24833200674298be3bb4c13716d4ef</t>
-  </si>
-  <si>
-    <t>ed4cff78d8d84760a6a2ac08df289333</t>
-  </si>
-  <si>
-    <t>ed64151c990c4fdabe6b7a7d0d3a05ff</t>
-  </si>
-  <si>
-    <t>ed64213272454f89a2f6195ef8d7eee7</t>
-  </si>
-  <si>
-    <t>edbeff155d46436d8194bddda0b47a48</t>
-  </si>
-  <si>
-    <t>edc30d423855472fa847bab9efe4ae15</t>
-  </si>
-  <si>
-    <t>ee445470b37047b49ed057143aa4d27e</t>
-  </si>
-  <si>
-    <t>ee7a334fdd284fdba60a47562cf56c48</t>
-  </si>
-  <si>
-    <t>eff35e16bc124333b7ea918c8c78e328</t>
-  </si>
-  <si>
-    <t>effa475431a748c49abf59f9d24afe6e</t>
-  </si>
-  <si>
-    <t>f026d14fa86748a19b94034bf8ac8256</t>
-  </si>
-  <si>
-    <t>f05e3ab9a4a048b79d41259aa494e77c</t>
-  </si>
-  <si>
-    <t>f1213f3c80f940a0bd6ffb27e3268cc5</t>
-  </si>
-  <si>
-    <t>f1819109579947ebba1c34be3ceb5d59</t>
-  </si>
-  <si>
-    <t>f1a52881bb154cf095204ed8661a9fbc</t>
-  </si>
-  <si>
-    <t>f1b920046a034482bfc7bb995315788f</t>
-  </si>
-  <si>
-    <t>f26594bd8b034d5cb5ac5746958fbba3</t>
-  </si>
-  <si>
-    <t>f2b2cecf7df74e5d82b18628df0d2f6a</t>
-  </si>
-  <si>
-    <t>f2d6d9b76de7428b886e4e8bbed9f9ea</t>
-  </si>
-  <si>
-    <t>f2dd4825d5294e198f22426b17734b99</t>
-  </si>
-  <si>
-    <t>f307bb53290e4aaf9d73fd0c1877ff14</t>
-  </si>
-  <si>
-    <t>f319f50b5e574e46862175f2dff6c769</t>
-  </si>
-  <si>
-    <t>f376d72a79fe4f48a1a16c9ac3bb3dc0</t>
-  </si>
-  <si>
-    <t>f5650c16daad48c4b13af252b374d053</t>
-  </si>
-  <si>
-    <t>f62fdbc9a8fd4ff6b041187cdcb5bed4</t>
-  </si>
-  <si>
-    <t>f6eb8d79ca0346e3a8c7b4e64d94eb22</t>
-  </si>
-  <si>
-    <t>f6fb731dce2a47b9b4d59f8ab15bb20d</t>
-  </si>
-  <si>
-    <t>f82dde7fc4db43578489548d4b949a1f</t>
-  </si>
-  <si>
-    <t>f83feff1d58a4d11ada839d85e6d6398</t>
-  </si>
-  <si>
-    <t>f8511a10713743e4ab85c3ce99bdda38</t>
-  </si>
-  <si>
-    <t>f85845c52af44f39a45e34f477ad925b</t>
-  </si>
-  <si>
-    <t>f85bb609cc484b9394cc68f22a82ccaf</t>
-  </si>
-  <si>
-    <t>f88472a74c124033a658c115c7ffe895</t>
-  </si>
-  <si>
-    <t>f8cc38939e21476d817d47f3672f34d3</t>
-  </si>
-  <si>
-    <t>f8e035b836b245a6b9fd2cf110aeb0c3</t>
-  </si>
-  <si>
-    <t>f93621b1bab54cd4bcc78ace4a884f5d</t>
-  </si>
-  <si>
-    <t>f944ea5ca1da4d109f5454265ad7e0bc</t>
-  </si>
-  <si>
-    <t>f9489cd74f7d45adb4abcb6eb97dbaf8</t>
-  </si>
-  <si>
-    <t>f9976ea724c24f429708fa57aa78dd77</t>
-  </si>
-  <si>
-    <t>faa6f1aa5bf545579cebee0eef057951</t>
-  </si>
-  <si>
-    <t>fab4e210483d4ff1a1c8eb81570d2970</t>
-  </si>
-  <si>
-    <t>fb673a1c66754db6945c63ffcdfab134</t>
-  </si>
-  <si>
-    <t>fbd710d469754ef0bb856c97bc94925c</t>
-  </si>
-  <si>
-    <t>fc80c852c2bd462ea7239268bb7ede6b</t>
-  </si>
-  <si>
-    <t>fd29fb786d404986acf455926b616e15</t>
-  </si>
-  <si>
-    <t>fd3c2df6cdfc406ab9c890c6ca414eb8</t>
-  </si>
-  <si>
-    <t>fd3fa18b62a54079b316f4dc5e5f26ad</t>
-  </si>
-  <si>
-    <t>fd8039176ee4444994c8b27c64f9f714</t>
-  </si>
-  <si>
-    <t>fdd96c7f2ea0479f857232982790b375</t>
-  </si>
-  <si>
-    <t>fe72fa7c7c5c406cb43064495e0932e4</t>
-  </si>
-  <si>
-    <t>feab66efd24a4d0c9cd1205abef9e006</t>
-  </si>
-  <si>
-    <t>fee28d2a86bf4284ab30372c0ef3fefc</t>
-  </si>
-  <si>
-    <t>ff3075c1b5b14b16a9e08868448bde2e</t>
-  </si>
-  <si>
-    <t>ffe7136104164f24b56165f9f8c0b274</t>
+    <t>0024e8d19559439a9cfcdf57790d0cdc</t>
+  </si>
+  <si>
+    <t>0034af1e338e49d0b2829a1763c22cda</t>
+  </si>
+  <si>
+    <t>00495c9882cd43f78ae26ca333f8625d</t>
+  </si>
+  <si>
+    <t>00626fd5731a4c5d814d76cc803f1c6e</t>
+  </si>
+  <si>
+    <t>00675865d7774e63b79b648aec254033</t>
+  </si>
+  <si>
+    <t>00afba42c3724392a4c9c2bce0b89162</t>
+  </si>
+  <si>
+    <t>00e820eea7db44f0835ca79f45a453ea</t>
+  </si>
+  <si>
+    <t>0114df4932c7482e9eab1d9f0873c015</t>
+  </si>
+  <si>
+    <t>012a68f63b9344baba47a18f0e9957bb</t>
+  </si>
+  <si>
+    <t>012d8807762a45b6bbb022a76cfed2bb</t>
+  </si>
+  <si>
+    <t>013c338c049646f585f928219ab123c8</t>
+  </si>
+  <si>
+    <t>014122a6b74d4fbe98621f9600c23d65</t>
+  </si>
+  <si>
+    <t>0209c76e5576427bbfeae65a21f40d7b</t>
+  </si>
+  <si>
+    <t>0219eebb38aa42998bf1de5f6fcdf305</t>
+  </si>
+  <si>
+    <t>034dce49ee564740a0343649a0a8ca2b</t>
+  </si>
+  <si>
+    <t>035067cd6ba741a08b3c2cae050f2957</t>
+  </si>
+  <si>
+    <t>037ab6064f3840058d6a13b400da5a0b</t>
+  </si>
+  <si>
+    <t>03b8e90627554006ade7ed88a7116a9d</t>
+  </si>
+  <si>
+    <t>04ed831baf1843e6ae79d5a8ad4f61fe</t>
+  </si>
+  <si>
+    <t>065c7b055efe400aae5805b56c14abd7</t>
+  </si>
+  <si>
+    <t>0667e5af733f49c3a8d56bdbc9eed7b9</t>
+  </si>
+  <si>
+    <t>0674405313d1483ca5ce98fba518e204</t>
+  </si>
+  <si>
+    <t>067ec6b634874bd1a49d60782935ee6e</t>
+  </si>
+  <si>
+    <t>069138c128d44de8b4c80db880dbdb3d</t>
+  </si>
+  <si>
+    <t>06ae684458114bf5a5d52d58ec3c8ffd</t>
+  </si>
+  <si>
+    <t>06cbc7af644542febf85e80cc877e3e8</t>
+  </si>
+  <si>
+    <t>06e7013ce3514392ad1b8d5de98d7df0</t>
+  </si>
+  <si>
+    <t>070435f9cfae49cea0ebee6d7c5ee907</t>
+  </si>
+  <si>
+    <t>0706ab253c07473bb841fc0d49d9b87a</t>
+  </si>
+  <si>
+    <t>076897a2a10740cc979c912d098768ed</t>
+  </si>
+  <si>
+    <t>078afeb639224bbf82f998a6f55be58a</t>
+  </si>
+  <si>
+    <t>07e1fc91f56a4f2cb071d231ecc7c922</t>
+  </si>
+  <si>
+    <t>08d1c5a740134a51b96f4f2d6d08e578</t>
+  </si>
+  <si>
+    <t>08db5cd292b24563973a1f7d33f8573e</t>
+  </si>
+  <si>
+    <t>0a5a2ed5ba2b4f1c8e64c7db2880a7c2</t>
+  </si>
+  <si>
+    <t>0a608e2321854d42ad211f0bec21bbd5</t>
+  </si>
+  <si>
+    <t>0a64dd0b694c4e3a962eb1e64c38c0a5</t>
+  </si>
+  <si>
+    <t>0ad4704ec83a4faf83cf4a5442069f38</t>
+  </si>
+  <si>
+    <t>0b6d42e89eac430a9fca0e4f57d13165</t>
+  </si>
+  <si>
+    <t>0ba10657e84c4d40aba6e63f1cf7da1b</t>
+  </si>
+  <si>
+    <t>0bd41136f1dc4a4fa1250ee115d632c6</t>
+  </si>
+  <si>
+    <t>0c1c1451ee8a4de78b0bbb0ef9e80437</t>
+  </si>
+  <si>
+    <t>0c2e575baa68474b8ac1fa8b8f2c1553</t>
+  </si>
+  <si>
+    <t>0c5843cd9eb04ccb962fe7e201e107e9</t>
+  </si>
+  <si>
+    <t>0c98b020b0d340a6ba7b8ec684a99335</t>
+  </si>
+  <si>
+    <t>0dbc7528e4374bf5a9ae680abbc6e61d</t>
+  </si>
+  <si>
+    <t>0f912536fe224bbcb0a9ea23e428a2ac</t>
+  </si>
+  <si>
+    <t>101b6926d33a4a4fb8c6ccd2e673e8a1</t>
+  </si>
+  <si>
+    <t>10433203e63645b2be0ead7a5b1e81a5</t>
+  </si>
+  <si>
+    <t>104c61f2432c4c42b582381607cb4b29</t>
+  </si>
+  <si>
+    <t>1079dcd45f6a44b2800e5e519c83a70b</t>
+  </si>
+  <si>
+    <t>112d262f16474216a43b7b7b49cb007c</t>
+  </si>
+  <si>
+    <t>1173a087a8a14847bc94cd41d4cd45dd</t>
+  </si>
+  <si>
+    <t>11895dbda75547bda4bf826fc99f78a0</t>
+  </si>
+  <si>
+    <t>1198423a44f148abb3ea2fc36d3cf624</t>
+  </si>
+  <si>
+    <t>1235d8edd3894061bf27b2941c77ac72</t>
+  </si>
+  <si>
+    <t>128a1cbbc59e432999d6bca75cf2f164</t>
+  </si>
+  <si>
+    <t>12ddf2533d4540ada616a6fa1b73765a</t>
+  </si>
+  <si>
+    <t>13055a9871c84413bdc82ee59a3a2b6a</t>
+  </si>
+  <si>
+    <t>13523861fb39430ba853964fd4402277</t>
+  </si>
+  <si>
+    <t>13a71dad997c47dc82befda4e706affe</t>
+  </si>
+  <si>
+    <t>13bcf2113ebf407bb06a834b2f11d439</t>
+  </si>
+  <si>
+    <t>13df61b1cd0e497abb2d7fe52d6ec23e</t>
+  </si>
+  <si>
+    <t>143fc20b721246b6a1d653b8bc3a26e7</t>
+  </si>
+  <si>
+    <t>15be185cd79b47599f6d66fc6cefa13f</t>
+  </si>
+  <si>
+    <t>162faedd3b4849a7911b23607e990869</t>
+  </si>
+  <si>
+    <t>1743e180b18e4d5aaad60a365b498a65</t>
+  </si>
+  <si>
+    <t>17b3972d59c24a109197c1ce41a8af8a</t>
+  </si>
+  <si>
+    <t>17dde0a414be48098a36210040219a54</t>
+  </si>
+  <si>
+    <t>18a7503a070241d196643606762c9f66</t>
+  </si>
+  <si>
+    <t>18c3f2cca23f4421a410822a373bdaf4</t>
+  </si>
+  <si>
+    <t>18fb4c88a3244d3ba274671b9d79c68c</t>
+  </si>
+  <si>
+    <t>18fc3e71570e4af685633fe5dd7b02eb</t>
+  </si>
+  <si>
+    <t>192c78b19e864f329725c501807a94cd</t>
+  </si>
+  <si>
+    <t>193fb92b48ee4632b03252857b63d0e4</t>
+  </si>
+  <si>
+    <t>1976986bb20e4ecd9af87c5bbdd41933</t>
+  </si>
+  <si>
+    <t>19eb848c8dc0465fae06e4aaa90ecd28</t>
+  </si>
+  <si>
+    <t>1b0ee2bb93fe43aa9ca38eecf2d07bd8</t>
+  </si>
+  <si>
+    <t>1b12754e354041339db2f9eeeffccb58</t>
+  </si>
+  <si>
+    <t>1b261d6ea98b40b5b6202b88193a1c7c</t>
+  </si>
+  <si>
+    <t>1b3b3d9ab6e749dc9fe4a91009a2a37a</t>
+  </si>
+  <si>
+    <t>1b8575a2dc1b415a809a7e3c0d9c826c</t>
+  </si>
+  <si>
+    <t>1c9522e02a7541dd959591819cd78b0b</t>
+  </si>
+  <si>
+    <t>1da3aff8fe2b4eb1ae6b2f7a631961ea</t>
+  </si>
+  <si>
+    <t>1db9942278504712b5e09fd6cc364b7a</t>
+  </si>
+  <si>
+    <t>1de25c80fbbd4cb69ba87b99cb31454d</t>
+  </si>
+  <si>
+    <t>1e5217d6da684c29adb408057a698786</t>
+  </si>
+  <si>
+    <t>203ad983b5d1493cae7f39099a7cc56d</t>
+  </si>
+  <si>
+    <t>2061cd0fd0ca499681e775d95d7c4893</t>
+  </si>
+  <si>
+    <t>2065155f3ba24f589e22368fae08e445</t>
+  </si>
+  <si>
+    <t>206f51c53c4e4881927e407aba93ca4c</t>
+  </si>
+  <si>
+    <t>20e53a4fc7c84122b85a8c1905f7f7f1</t>
+  </si>
+  <si>
+    <t>219c2a73cb0c47d4991a918940096cfb</t>
+  </si>
+  <si>
+    <t>21bd7ec315e64a7b98758fb398bc7db5</t>
+  </si>
+  <si>
+    <t>2205e881e4c945f7afc46400a3285254</t>
+  </si>
+  <si>
+    <t>2245f6603fae4700a28f37e7854acb77</t>
+  </si>
+  <si>
+    <t>2352abfab63c4de79a17f05f7b88f435</t>
+  </si>
+  <si>
+    <t>23688240760040dd92bd842f0636ebe1</t>
+  </si>
+  <si>
+    <t>236bec736f8645938d78e33abee1e5e1</t>
+  </si>
+  <si>
+    <t>23f0e80b31044f90b8d52fdbdabcd59c</t>
+  </si>
+  <si>
+    <t>2454dea2bce5430a9bdec97cd4391d7e</t>
+  </si>
+  <si>
+    <t>24803884b1b44e0589aeb33293f9cf77</t>
+  </si>
+  <si>
+    <t>248f997dadc54a17bc2e1566d7aa8b22</t>
+  </si>
+  <si>
+    <t>24c39bad27fc45029f0b8066c1e6589c</t>
+  </si>
+  <si>
+    <t>255137e45f044b879d5d2be93e0246c9</t>
+  </si>
+  <si>
+    <t>25d2337197644aaba6fd44527823fb03</t>
+  </si>
+  <si>
+    <t>269fbb85451b4d65b000427a67105a5a</t>
+  </si>
+  <si>
+    <t>26dc8f732fee4d749cf35bf0dff75c53</t>
+  </si>
+  <si>
+    <t>27134fed0abb403db2ec778382de6fa7</t>
+  </si>
+  <si>
+    <t>273c46ba71d64082885760b5d7349f51</t>
+  </si>
+  <si>
+    <t>274b310a71944d97923f963832d22fed</t>
+  </si>
+  <si>
+    <t>27681fc9fa0c48ab9fbdb736aba4f44f</t>
+  </si>
+  <si>
+    <t>277ffbbbadad466ca360ed7adc6a8196</t>
+  </si>
+  <si>
+    <t>2806ed4b4bc5472aacb29aca71f08739</t>
+  </si>
+  <si>
+    <t>280ba54a1960427c8f2d7a43637bdcff</t>
+  </si>
+  <si>
+    <t>2820cb049e22447684316b5036cdba80</t>
+  </si>
+  <si>
+    <t>2823a5c94c0c4617b64c3acf272a9940</t>
+  </si>
+  <si>
+    <t>2879118b166a4f89bf7bf75ddda0314e</t>
+  </si>
+  <si>
+    <t>29340b0083e5422f8e451b9927298d44</t>
+  </si>
+  <si>
+    <t>2a0f8ae3926b4733a0e0ddc45cb0e729</t>
+  </si>
+  <si>
+    <t>2a2395c9c0cb4fccb0982f3674527098</t>
+  </si>
+  <si>
+    <t>2ac28b4ccb7e4cd3a6e2e4e7556f8b51</t>
+  </si>
+  <si>
+    <t>2ad3c8e3b1eb4134a4a6592cbc221744</t>
+  </si>
+  <si>
+    <t>2b3982b4507c4c8a8c1306e273c4a419</t>
+  </si>
+  <si>
+    <t>2b75fe29fe464c8cbcd42a573f1b108c</t>
+  </si>
+  <si>
+    <t>2c008e94433c4a08834a848f91d0380b</t>
+  </si>
+  <si>
+    <t>2c2c71e4396e4194b914f6d77e090527</t>
+  </si>
+  <si>
+    <t>2cb569b341f04ed1ac33b8e71af3023e</t>
+  </si>
+  <si>
+    <t>2d1dd4409c40470ab1e8589d7349bee4</t>
+  </si>
+  <si>
+    <t>2d8a9e72f0f14bc098d04263bc275b25</t>
+  </si>
+  <si>
+    <t>2de4a40536c04c6ca9473e16d8a13db9</t>
+  </si>
+  <si>
+    <t>2e461212a7a54c94b4b2be983f4f1941</t>
+  </si>
+  <si>
+    <t>2ead7597bb784bfdabeddf530df40430</t>
+  </si>
+  <si>
+    <t>2ebc39d8fc9a4a65ad1265f68eb45f06</t>
+  </si>
+  <si>
+    <t>30437e2d404048db8e9a3b7a1524fc5f</t>
+  </si>
+  <si>
+    <t>30eaedd187c0486e9bf100a5858b2bba</t>
+  </si>
+  <si>
+    <t>30f7d2a6e86d4631865195b9ce231437</t>
+  </si>
+  <si>
+    <t>3108ad1cd98b46d1a04f0698291b3b3c</t>
+  </si>
+  <si>
+    <t>31320e2a02f140dfb39758b6594a85ff</t>
+  </si>
+  <si>
+    <t>31406472e2dd4597b8935ec4df1454e5</t>
+  </si>
+  <si>
+    <t>31bd05c8406544498b2440a28eef6f84</t>
+  </si>
+  <si>
+    <t>31e8067c39d74624b874620a81862ba2</t>
+  </si>
+  <si>
+    <t>325bb39d4bc546f8ac662da8f479c310</t>
+  </si>
+  <si>
+    <t>32692e0a4e9e44be8d4cb9263b115f1e</t>
+  </si>
+  <si>
+    <t>327d3feb95d043b0a2dfbe0af0aa95b5</t>
+  </si>
+  <si>
+    <t>32e2792ea2914616872f94ff5ef8fa1b</t>
+  </si>
+  <si>
+    <t>3325efb1db9241728cda4add2109d7fd</t>
+  </si>
+  <si>
+    <t>333b7453274a4384a1c0dbf044f9363e</t>
+  </si>
+  <si>
+    <t>33c0e928c0f944fd992551c1c15ab52d</t>
+  </si>
+  <si>
+    <t>33f3ad05a7f24298b0f7610a9e32bf7c</t>
+  </si>
+  <si>
+    <t>3460498960ec46ca9401f0cfab9b7da0</t>
+  </si>
+  <si>
+    <t>34d3e85f4da04ce7b3b678d47ae520d2</t>
+  </si>
+  <si>
+    <t>35476b2abb1d439a9764a085c72e3a15</t>
+  </si>
+  <si>
+    <t>355cf8c103214eaca49c98538db84d02</t>
+  </si>
+  <si>
+    <t>355e147c178d4a4b9d26f010994d0b1d</t>
+  </si>
+  <si>
+    <t>35719da73d9c4c73990837c7167cd48f</t>
+  </si>
+  <si>
+    <t>35e92232a498447da951cb6a78d2acd6</t>
+  </si>
+  <si>
+    <t>35ef68635e674d878e43b1d5a33578b4</t>
+  </si>
+  <si>
+    <t>369a020e8403459a9d4d54bdb9a42d8d</t>
+  </si>
+  <si>
+    <t>370c5901b6ef4fa0ad963a4a219edd35</t>
+  </si>
+  <si>
+    <t>3726b9f3e2b7480a9e03d2b1ce05b7c5</t>
+  </si>
+  <si>
+    <t>3751abf4edc242e5a8974b620ea74e24</t>
+  </si>
+  <si>
+    <t>37a677e4a8df4d2992ec4494eebeb2d7</t>
+  </si>
+  <si>
+    <t>37ae2846d20b4a3c9b6b3490e78240a5</t>
+  </si>
+  <si>
+    <t>38d03efeccb84290a20076eae849cc80</t>
+  </si>
+  <si>
+    <t>38d5d03db77a47fc9c265a5643a4cb86</t>
+  </si>
+  <si>
+    <t>39021127527a465285c187d6878c2b23</t>
+  </si>
+  <si>
+    <t>3949b1b29e684f0fbf833e22d68dc17c</t>
+  </si>
+  <si>
+    <t>39eaa6b91186456b9e153c0119733eb1</t>
+  </si>
+  <si>
+    <t>3a1380d2cfa3491083f6ed707935b10d</t>
+  </si>
+  <si>
+    <t>3a1df470126540f9af10ea6ad4688e70</t>
+  </si>
+  <si>
+    <t>3a2260432b404d42aa82de7bd29a628e</t>
+  </si>
+  <si>
+    <t>3a63a376248a4067af0290cb6d177096</t>
+  </si>
+  <si>
+    <t>3aa21e24c01c45eabe719ca1e07354b5</t>
+  </si>
+  <si>
+    <t>3aa75ad984954e9f8ff49bab7fdbfaac</t>
+  </si>
+  <si>
+    <t>3accc238583e4d6dbbf65f5ba74dd6eb</t>
+  </si>
+  <si>
+    <t>3b4e988dc96d4d08bcf81f9ed5c3d978</t>
+  </si>
+  <si>
+    <t>3bd4fefcf946464793ffb6df82c0a280</t>
+  </si>
+  <si>
+    <t>3c03d56a95664c488585d93ebae92163</t>
+  </si>
+  <si>
+    <t>3c0a5f6d92714c489e90538502cd0b7c</t>
+  </si>
+  <si>
+    <t>3c18f8b581e44255a7ae1492b3ca863b</t>
+  </si>
+  <si>
+    <t>3c1b73e725f94f8f9ea58f6bc5362250</t>
+  </si>
+  <si>
+    <t>3cba659cc9de46349e6a90eed2caec68</t>
+  </si>
+  <si>
+    <t>3cf1b60061654f5eb0307edc0ae68076</t>
+  </si>
+  <si>
+    <t>3d41a72c07d14a188d13ca94976079a2</t>
+  </si>
+  <si>
+    <t>3d5911f8007a4cc588591951419a11f8</t>
+  </si>
+  <si>
+    <t>3d6160b8bf164320a839dc58718a43c6</t>
+  </si>
+  <si>
+    <t>3d8442f2a8db4953875b7a356f837f6c</t>
+  </si>
+  <si>
+    <t>3defd8b4431243a6b4f5fad59963bdce</t>
+  </si>
+  <si>
+    <t>3e28c1a407f74429940d43e2ee8e772c</t>
+  </si>
+  <si>
+    <t>3e2f2da18f3741d89dfc806fb172df60</t>
+  </si>
+  <si>
+    <t>3eaa588ffed64ba0b76cc8fd3633c0c1</t>
+  </si>
+  <si>
+    <t>3edbc39aa5ca4f1796777b562c4b4fad</t>
+  </si>
+  <si>
+    <t>3f54b54ddebb4b26bd00bad030138702</t>
+  </si>
+  <si>
+    <t>3f88d886f35e4f55a0fceea82d17b4d7</t>
+  </si>
+  <si>
+    <t>3f8d8297efd64bdaa3ecfdbdbb674ae0</t>
+  </si>
+  <si>
+    <t>3f98549085ff46aba39b7ca8986f2e37</t>
+  </si>
+  <si>
+    <t>3fad50e9889f49f39bb62003737b9201</t>
+  </si>
+  <si>
+    <t>3fcc6091a5ed44f1a7213c6571db1ef7</t>
+  </si>
+  <si>
+    <t>3fe39ae806124311ac838b5c040f64ea</t>
+  </si>
+  <si>
+    <t>4012d9bafeb445efbf3751f13342f6a9</t>
+  </si>
+  <si>
+    <t>401bd25448dd4fe1ac5a64b10dbb218b</t>
+  </si>
+  <si>
+    <t>40420736807a4f81b4f7ddab97fb0351</t>
+  </si>
+  <si>
+    <t>407d00209d2b42ec8528c7a3e730b1ed</t>
+  </si>
+  <si>
+    <t>4080cd8f969440a4a0e2e85f4667cbfc</t>
+  </si>
+  <si>
+    <t>409f3b7ea05e45f79afd4c2b365ea693</t>
+  </si>
+  <si>
+    <t>4137dc089fdf47d18490ca76bcdb786b</t>
+  </si>
+  <si>
+    <t>41409b76faae40a2b9a8699ba7a4ea09</t>
+  </si>
+  <si>
+    <t>4147959f7fd2499b95885f52f21852ba</t>
+  </si>
+  <si>
+    <t>418929712d824b9698728da5b8cbf297</t>
+  </si>
+  <si>
+    <t>41906ed00ac04a2ebbf072afae34940d</t>
+  </si>
+  <si>
+    <t>419f7700b3554b10980123629e0b6b58</t>
+  </si>
+  <si>
+    <t>423c40b55f8e4035b00ee2afdd939793</t>
+  </si>
+  <si>
+    <t>42624d67eca2452180b9b807ffd67d6f</t>
+  </si>
+  <si>
+    <t>4276c5857d7e42199b5dc4f11fbbaa06</t>
+  </si>
+  <si>
+    <t>42ecfcebd25e450689a44ad3e380ec68</t>
+  </si>
+  <si>
+    <t>43056389dc934445bf7e89fbc9b9bcf9</t>
+  </si>
+  <si>
+    <t>43633c65d8d34131b6130d4de0fe683b</t>
+  </si>
+  <si>
+    <t>438876389e504d218d183c1d5b93e158</t>
+  </si>
+  <si>
+    <t>43ae87d58f294930b5137dc515d80335</t>
+  </si>
+  <si>
+    <t>4406f9e7327e4a438c2bcf0a7aea6099</t>
+  </si>
+  <si>
+    <t>4449529a8c3541188c03b7c133002c75</t>
+  </si>
+  <si>
+    <t>4477acbe04e647e4b17704f1e177c7e1</t>
+  </si>
+  <si>
+    <t>45bfa0c9d02c41518a93d63eced100f5</t>
+  </si>
+  <si>
+    <t>4608ad18a3bf4fd5a7e54dc889bef95b</t>
+  </si>
+  <si>
+    <t>464799d2db1a42d4bdad459c025af364</t>
+  </si>
+  <si>
+    <t>46e277e1d2b544da8d99dee09bb23023</t>
+  </si>
+  <si>
+    <t>46f24df714da478688dd4f0f0057f1e4</t>
+  </si>
+  <si>
+    <t>470514f1fa984e1a92cbb11994959a28</t>
+  </si>
+  <si>
+    <t>470d3b314dde4c9d84a2dda14f660676</t>
+  </si>
+  <si>
+    <t>4725a0d35e724dcb8375b2b3a29af5c9</t>
+  </si>
+  <si>
+    <t>473733cfae754b5bbc77c78aaba54b37</t>
+  </si>
+  <si>
+    <t>4786f2c3b7694c73a0622e04b371f215</t>
+  </si>
+  <si>
+    <t>483a3c790c8a4f7694b70fd8bc277010</t>
+  </si>
+  <si>
+    <t>49b03513d29b48bb91843e9876e32395</t>
+  </si>
+  <si>
+    <t>49f83be4008141dd916c1a995c27ebce</t>
+  </si>
+  <si>
+    <t>4ac0cb8318084f908f1f9f7ad3f95857</t>
+  </si>
+  <si>
+    <t>4b8ce8b4347248eeac0344914bb2df65</t>
+  </si>
+  <si>
+    <t>4c1db23337944c1095a911ba0842dedb</t>
+  </si>
+  <si>
+    <t>4c24734f50e048f8b35a4bac047c321a</t>
+  </si>
+  <si>
+    <t>4c91ed9e4b244ddc9d5a6243dcb864af</t>
+  </si>
+  <si>
+    <t>4c9f99d20c3649f5821b6d75e058b364</t>
+  </si>
+  <si>
+    <t>4cc9310af44e47c9823d97935b3efc02</t>
+  </si>
+  <si>
+    <t>4cd171c39a1244f6ba67f9e09168c6ee</t>
+  </si>
+  <si>
+    <t>4d9c2d54c6a64e9a92699a2dccf7da18</t>
+  </si>
+  <si>
+    <t>4ebed5fe249b43b4848f92b84593b029</t>
+  </si>
+  <si>
+    <t>4ec3ab6f84c944e7ba24a5a9a0cd812a</t>
+  </si>
+  <si>
+    <t>4eee981e82ef4387968bd00edd4f39be</t>
+  </si>
+  <si>
+    <t>4eefcb32ad1d44a0898208018e9e4f78</t>
+  </si>
+  <si>
+    <t>4f174d61130442a78b8a140aa0c40b66</t>
+  </si>
+  <si>
+    <t>4f41d0f4d80b4812b8e241961330d812</t>
+  </si>
+  <si>
+    <t>4f48122d8d3b4a41a600370fc2464a60</t>
+  </si>
+  <si>
+    <t>4f68229dcd1b4d20a3cc7d322573a1af</t>
+  </si>
+  <si>
+    <t>504beeee0af743e094ca1eb59c4c0081</t>
+  </si>
+  <si>
+    <t>508087bc8ec74388b6a65c44f170a970</t>
+  </si>
+  <si>
+    <t>50e6d86fef944be68228980dae22ee48</t>
+  </si>
+  <si>
+    <t>510a0545155441b69989a0283e02ecd5</t>
+  </si>
+  <si>
+    <t>51120cf8760d4bbd8b8c5330451fc46f</t>
+  </si>
+  <si>
+    <t>5137ad3733d345f7ba1de168dafaf233</t>
+  </si>
+  <si>
+    <t>51b2d21627cc4bf1b615d0bf702a1356</t>
+  </si>
+  <si>
+    <t>5202d406abe5442ba9d3df9531ae7bb6</t>
+  </si>
+  <si>
+    <t>524f989fbdf94e02ac73c0494a873c4c</t>
+  </si>
+  <si>
+    <t>52530cff3777426cbacd5dbc04bad220</t>
+  </si>
+  <si>
+    <t>52d8be8553fa46659b2c7c152a17a4be</t>
+  </si>
+  <si>
+    <t>532ce1b3082944e1832ee406e903d4a5</t>
+  </si>
+  <si>
+    <t>534ef75906df4222a57a340e5e5159c5</t>
+  </si>
+  <si>
+    <t>5411b03e79ac4ba5b681b39adb574f5d</t>
+  </si>
+  <si>
+    <t>54596760366b48ee8b976420659cb0f7</t>
+  </si>
+  <si>
+    <t>5462011528424c29ac706a9df206037d</t>
+  </si>
+  <si>
+    <t>546d9feb158345638f9299b9bf71653f</t>
+  </si>
+  <si>
+    <t>54e74c6f223848a3817092aeecb96d0c</t>
+  </si>
+  <si>
+    <t>5551916964324432b958a69772d777aa</t>
+  </si>
+  <si>
+    <t>5553039635f74b06b186bb1d495c8bb0</t>
+  </si>
+  <si>
+    <t>55aa3f163c724c79a71f55059b112b17</t>
+  </si>
+  <si>
+    <t>566ee797dd994f0792d265ea047c88b5</t>
+  </si>
+  <si>
+    <t>56b5f04a7fb7409381257175292a6acf</t>
+  </si>
+  <si>
+    <t>56d7f6385b10443da3ccfbd59684baae</t>
+  </si>
+  <si>
+    <t>578747c7369245e69563bad82388a018</t>
+  </si>
+  <si>
+    <t>57c883e453d14a97805aaaa83187feef</t>
+  </si>
+  <si>
+    <t>582a09cedf8a460996aabca0c2385e7a</t>
+  </si>
+  <si>
+    <t>5845d8ff96b248b48344b53ef2ad2755</t>
+  </si>
+  <si>
+    <t>58a8c2e1d22647cdbc74d7d363ee2b0b</t>
+  </si>
+  <si>
+    <t>591f6e6e8e3f423d92d287014bf5c248</t>
+  </si>
+  <si>
+    <t>593d358cdbf64136a304d2fdc8b6b106</t>
+  </si>
+  <si>
+    <t>5a275108a0e9484897a9581f34b9f223</t>
+  </si>
+  <si>
+    <t>5a452021fa28463aba55d6988e267e45</t>
+  </si>
+  <si>
+    <t>5a96f596e007484d813257cec369dc5b</t>
+  </si>
+  <si>
+    <t>5aed9997502349db99bb8814d96697fa</t>
+  </si>
+  <si>
+    <t>5b0c07c459c441c7b14c5f25babca7c8</t>
+  </si>
+  <si>
+    <t>5b4aa803586e47d9a6f8990cc7f18db0</t>
+  </si>
+  <si>
+    <t>5bb02a3978094ed9b5bb3d4a8b38e309</t>
+  </si>
+  <si>
+    <t>5bba4d5d2d1e4a0f8bd470be80f81a66</t>
+  </si>
+  <si>
+    <t>5bc1583c356d48f79949566956ba3816</t>
+  </si>
+  <si>
+    <t>5bf75aadb8c64d5fb5a16f27a5fd1c4d</t>
+  </si>
+  <si>
+    <t>5c0f1bf042c14a22aed4574b336e61b9</t>
+  </si>
+  <si>
+    <t>5c3595e829994e33ad0fc442fc945882</t>
+  </si>
+  <si>
+    <t>5c5707ccd7ae439387642f34608b5d30</t>
+  </si>
+  <si>
+    <t>5d274b0f4c504104ab3a19e7994128e5</t>
+  </si>
+  <si>
+    <t>5e0466d5c4ed42a1bc266cb1ab369cb9</t>
+  </si>
+  <si>
+    <t>5e0b1cdbba1a47489cb7d85676c59936</t>
+  </si>
+  <si>
+    <t>5e2e92f140714869b4035effa91b78d2</t>
+  </si>
+  <si>
+    <t>5e6b6b4d1c8a4c5f94f526e5698f56e7</t>
+  </si>
+  <si>
+    <t>5e8ebdf4b6f64acb9d7743a9b7c6c717</t>
+  </si>
+  <si>
+    <t>5eff1a2a652d471486d291d377ff60f2</t>
+  </si>
+  <si>
+    <t>5fa7747cd90a4badab0d889714eafc4b</t>
+  </si>
+  <si>
+    <t>5faebcd987384d6d9974c99fb36f719d</t>
+  </si>
+  <si>
+    <t>604424f4ebe74099ac301a8ab248e5b6</t>
+  </si>
+  <si>
+    <t>605a242930f64ee791169110e7458dd0</t>
+  </si>
+  <si>
+    <t>61946d2469ea45b1b1de19e25d81ac99</t>
+  </si>
+  <si>
+    <t>61d137b7cc9e4f68a1ba37ad98e8caec</t>
+  </si>
+  <si>
+    <t>626b399d853f4e7abd2ea3d8e864bcb7</t>
+  </si>
+  <si>
+    <t>62a57c67f1c642eb9f3e049312efd809</t>
+  </si>
+  <si>
+    <t>62d82061841d4dfaabec41b3c0457719</t>
+  </si>
+  <si>
+    <t>62ed4089145d4d6a8456a3dadaa96bd6</t>
+  </si>
+  <si>
+    <t>62f32b9bf58c40b4888e5f71bffec14c</t>
+  </si>
+  <si>
+    <t>630f842a60724cfdb96e8e0c3d395d49</t>
+  </si>
+  <si>
+    <t>636a4dfe97dd44caaac57ee1a180d98b</t>
+  </si>
+  <si>
+    <t>6374253279654d9db9273d00d944fd80</t>
+  </si>
+  <si>
+    <t>63f1ffc6aea243edb7c01dff96ed96c1</t>
+  </si>
+  <si>
+    <t>64151985b5b9402cbc5b2844dc7260d9</t>
+  </si>
+  <si>
+    <t>641a02db1d4f47fdb660ee0bea16cbe0</t>
+  </si>
+  <si>
+    <t>6526485c3f25489fbc33893607decc69</t>
+  </si>
+  <si>
+    <t>652e8bd1266044889fa93f8e8f73b9b0</t>
+  </si>
+  <si>
+    <t>65819d22c09142619be47edaed6922ad</t>
+  </si>
+  <si>
+    <t>65c902d3cf3d45b591e9209e4bcbb819</t>
+  </si>
+  <si>
+    <t>668770984f7c43de9c8189ebd6f2e517</t>
+  </si>
+  <si>
+    <t>66989f15444544149c745ee80be7d2de</t>
+  </si>
+  <si>
+    <t>66b1d01ad04b455d97ee731cd26aee41</t>
+  </si>
+  <si>
+    <t>66bc2e70f2814088a791c506214f9585</t>
+  </si>
+  <si>
+    <t>66dd30dad8704c2fb46be7ef7012da3d</t>
+  </si>
+  <si>
+    <t>66ffb8b4192c4faf80e839d7054a652e</t>
+  </si>
+  <si>
+    <t>675621a616274cecaac0d9b204ae765f</t>
+  </si>
+  <si>
+    <t>679b32166f3e48aa909d3832402cb36d</t>
+  </si>
+  <si>
+    <t>67f0ebac6f3f4fe1aaea8c216b637314</t>
+  </si>
+  <si>
+    <t>68b2a8a7eef44eb3a033f453cda59690</t>
+  </si>
+  <si>
+    <t>68fa929445b149c6b44273e8f5d2e8fb</t>
+  </si>
+  <si>
+    <t>693c741c9199428895b2b8847829c417</t>
+  </si>
+  <si>
+    <t>694c441e72d24fa591ec76dab29d4dd6</t>
+  </si>
+  <si>
+    <t>695720d481594637ac0c7f463558ed7e</t>
+  </si>
+  <si>
+    <t>69dea7667e6649529677e54644641bac</t>
+  </si>
+  <si>
+    <t>6a021cde0d24465ca30171cb393f6099</t>
+  </si>
+  <si>
+    <t>6a21f41afb924259b50e1a969130913e</t>
+  </si>
+  <si>
+    <t>6a259766fb26415a938ff20f2c964d4e</t>
+  </si>
+  <si>
+    <t>6a47e70a569c43d8a39ad19abc726ba5</t>
+  </si>
+  <si>
+    <t>6a832c78c01c4bbaad9a93d71f3c2bd0</t>
+  </si>
+  <si>
+    <t>6a9fd84fd82e4eebac057e03dda40630</t>
+  </si>
+  <si>
+    <t>6ac1372f433349b38611d846f34be8d0</t>
+  </si>
+  <si>
+    <t>6aeb3cfec01c430195ef99620cce01bb</t>
+  </si>
+  <si>
+    <t>6afde7dd05be46bca67ce69d147714ee</t>
+  </si>
+  <si>
+    <t>6b01c69e38194ed28809e9cd350cba8d</t>
+  </si>
+  <si>
+    <t>6b0452f0a97241a68251cf9cc5c0ffd5</t>
+  </si>
+  <si>
+    <t>6b49a3bd193e4fc1b1467d17323e489d</t>
+  </si>
+  <si>
+    <t>6ba226dcf38a4216b8c554b31914076c</t>
+  </si>
+  <si>
+    <t>6c4597c8acd84492acc7ccaf1bedb489</t>
+  </si>
+  <si>
+    <t>6c4dcf3b88b94ef6ac4a65e3f9ccb46b</t>
+  </si>
+  <si>
+    <t>6c5aabfae7a74c1a8b8c157c521da778</t>
+  </si>
+  <si>
+    <t>6cd3bf3f50684a5f9278ebb7ddba01eb</t>
+  </si>
+  <si>
+    <t>6d783ad4402e46f99d571bc2fd020690</t>
+  </si>
+  <si>
+    <t>6eba3f03e6b64a49a89d4328da4c906a</t>
+  </si>
+  <si>
+    <t>6ec7d0df9c3b4a5faddcf848cc87ef5a</t>
+  </si>
+  <si>
+    <t>6f19f342118f4935a0540c30a4b12f7a</t>
+  </si>
+  <si>
+    <t>6f514140444b49b49f2db4dab8ef8546</t>
+  </si>
+  <si>
+    <t>6fe8bd494b1944939ff77f1b7abf28cb</t>
+  </si>
+  <si>
+    <t>70417d3790a242249b59c5a17e5186c4</t>
+  </si>
+  <si>
+    <t>706eef785f4f44a2ab79ad20f405745f</t>
+  </si>
+  <si>
+    <t>70781efffdc1473fa15a00c1b7d629af</t>
+  </si>
+  <si>
+    <t>70f7513ff59245439356f748da4eb6a4</t>
+  </si>
+  <si>
+    <t>7165c59f76434e26a35f28891f2ed465</t>
+  </si>
+  <si>
+    <t>71f5d97d161d4ffea0032cd70eb1e318</t>
+  </si>
+  <si>
+    <t>71f646c3f9034c69ad7c39a29d2d297f</t>
+  </si>
+  <si>
+    <t>722066406f6141e182d34fb561e6a99d</t>
+  </si>
+  <si>
+    <t>72e45b61b6b74ff2ba9d6d5d463a5fd1</t>
+  </si>
+  <si>
+    <t>73ae52937aa54a63a0c978dd9dc0429a</t>
+  </si>
+  <si>
+    <t>73cd15eddc5b4222b06f38480f7a57cf</t>
+  </si>
+  <si>
+    <t>7423bb7fd3214c598e710f10a1fac9ab</t>
+  </si>
+  <si>
+    <t>746fbef61a374607b2fe31e4bd2a0b6e</t>
+  </si>
+  <si>
+    <t>74c7bda95f0c402abc06484880b12465</t>
+  </si>
+  <si>
+    <t>74e625854f07439e97bed934dbca1adf</t>
+  </si>
+  <si>
+    <t>7613214ac005451c93bb4027c9195bbf</t>
+  </si>
+  <si>
+    <t>7613c908e3d348a983519c85222313a4</t>
+  </si>
+  <si>
+    <t>7621f7dc0b584c6789592f175d26d3c8</t>
+  </si>
+  <si>
+    <t>763ecf1052e64af1bfce9dd6c023770f</t>
+  </si>
+  <si>
+    <t>76a40f3cc61144bb8dcd8a6268ab6439</t>
+  </si>
+  <si>
+    <t>76ffe7403e344af98e03b62a9acd26df</t>
+  </si>
+  <si>
+    <t>77544ff917e4462b939a9e0bc2996cf8</t>
+  </si>
+  <si>
+    <t>784d8bf02e67427a821e876c11a8031f</t>
+  </si>
+  <si>
+    <t>78cd69933d0b4ae69daaba6a03837a19</t>
+  </si>
+  <si>
+    <t>78e8aba4b5174392b120ccb715959e9b</t>
+  </si>
+  <si>
+    <t>7908714ea3ae409d9b6cdfc602ef6a33</t>
+  </si>
+  <si>
+    <t>794ad569da5f47b7ba19fef6f3cc2b35</t>
+  </si>
+  <si>
+    <t>7a184bef7fe14c5d8d748fec0c7d3ddd</t>
+  </si>
+  <si>
+    <t>7a53907993264680af8e81492c979541</t>
+  </si>
+  <si>
+    <t>7a66577178484fe3a9097a38fb1193ae</t>
+  </si>
+  <si>
+    <t>7ae0b795c4ea4ec780c02d5faab82a15</t>
+  </si>
+  <si>
+    <t>7b5b0ee2013e45c690f887bdb2757eda</t>
+  </si>
+  <si>
+    <t>7b778aff623749f48e21847024c8ce44</t>
+  </si>
+  <si>
+    <t>7bcf14c9643146208bf94b0ba50481b1</t>
+  </si>
+  <si>
+    <t>7bd3915f56ec44c7a01e0f88a1b65c22</t>
+  </si>
+  <si>
+    <t>7c636919741f4f46b0f491c40cb0a314</t>
+  </si>
+  <si>
+    <t>7c90f0b50a554054a7ee48281b3a9ce4</t>
+  </si>
+  <si>
+    <t>7c9bda3cb2844803a1772b2184b70161</t>
+  </si>
+  <si>
+    <t>7d01d7d43d1241a585e97b3c68289af8</t>
+  </si>
+  <si>
+    <t>7d49c0a0d59a4699aad1c315e7286248</t>
+  </si>
+  <si>
+    <t>7d8fb786c10e4aa4b715f51f7261eaa0</t>
+  </si>
+  <si>
+    <t>7dab31a3fc054903a028fe642fe82645</t>
+  </si>
+  <si>
+    <t>7e9e0d0834e646c4bc122db0f3d71c49</t>
+  </si>
+  <si>
+    <t>7ebb8cc759a14476914db4c479903fbb</t>
+  </si>
+  <si>
+    <t>7f7d334c7a9c443d849552482bcc2f2d</t>
+  </si>
+  <si>
+    <t>7fa7b7a6ea17413a841e4ec9a642722a</t>
+  </si>
+  <si>
+    <t>7fdfc48992414ea5ab7b2f8721830615</t>
+  </si>
+  <si>
+    <t>805c2def672d4bbabacaff6a8615294f</t>
+  </si>
+  <si>
+    <t>806e14ec05c647ad9c9c1f0db26902e6</t>
+  </si>
+  <si>
+    <t>806f91efbe6047e9bb92807b054640af</t>
+  </si>
+  <si>
+    <t>80d9edb8d149420cb0de348004a5b87f</t>
+  </si>
+  <si>
+    <t>81c95caf9e114fcba32f5a627a12f42d</t>
+  </si>
+  <si>
+    <t>8292f5ddd8214a4ab20c26b11820f0d7</t>
+  </si>
+  <si>
+    <t>82b9a1777b2c4c4a867a2d56dc469697</t>
+  </si>
+  <si>
+    <t>82fdd346be724ce692dba3d7123e0d6e</t>
+  </si>
+  <si>
+    <t>843763108978400b901d6bf36b00d913</t>
+  </si>
+  <si>
+    <t>8467b8a4ad984d1b8b32e87a50ba2622</t>
+  </si>
+  <si>
+    <t>85650d9bdec9408e8fc8890c036911ca</t>
+  </si>
+  <si>
+    <t>870196e402ee48259df90ab4d8af8209</t>
+  </si>
+  <si>
+    <t>8730e8db19a444c697335aedb5610120</t>
+  </si>
+  <si>
+    <t>8740fa3bcda845a9a79d5fdd2fb427bf</t>
+  </si>
+  <si>
+    <t>87788d636dac4e118208a8307ea77d26</t>
+  </si>
+  <si>
+    <t>877c6409b01348569df7d1a52cf9f611</t>
+  </si>
+  <si>
+    <t>87c9875ca28a4f00a4589c2f1469ce78</t>
+  </si>
+  <si>
+    <t>88226092880645069fc3743a43a93c77</t>
+  </si>
+  <si>
+    <t>88338fa3d72842f8ac387e14b910f46c</t>
+  </si>
+  <si>
+    <t>885fe31a9a584fd38fa5fde6d7903166</t>
+  </si>
+  <si>
+    <t>89066b034ead414198ae84e489f2055d</t>
+  </si>
+  <si>
+    <t>893b8d93aacd4c37a44fd67c766356e8</t>
+  </si>
+  <si>
+    <t>8995c22d4e0d4ea99834370d6a542c0c</t>
+  </si>
+  <si>
+    <t>8a736bc490814b4eb605cb19e1f71f42</t>
+  </si>
+  <si>
+    <t>8a78c57a75f54518aed1aac1d87435ce</t>
+  </si>
+  <si>
+    <t>8a8d42312ba940c3ab84ba082161efbc</t>
+  </si>
+  <si>
+    <t>8ad0aad6954a4468a1bd55ce6e828c43</t>
+  </si>
+  <si>
+    <t>8bec9095f93c40468a42cb8ee61493cd</t>
+  </si>
+  <si>
+    <t>8c38469d881641208fcc8ce0e43a137a</t>
+  </si>
+  <si>
+    <t>8cd4fe896a16488bb9ec1b2fae96c428</t>
+  </si>
+  <si>
+    <t>8d38534651e44b959d7f077f1df8a872</t>
+  </si>
+  <si>
+    <t>8d87eed0e06d40d29986ccbd7e2d7f05</t>
+  </si>
+  <si>
+    <t>8d9e405c97054e3a8af8f81e7353990e</t>
+  </si>
+  <si>
+    <t>8e96b5d9e24e4db29a572f5884173522</t>
+  </si>
+  <si>
+    <t>8eea060628974c4bb190049e8e96d689</t>
+  </si>
+  <si>
+    <t>8f1a876ac2144aabaf6dee3477de1a27</t>
+  </si>
+  <si>
+    <t>8f2763e9218e49aaa693f54cf2e424ef</t>
+  </si>
+  <si>
+    <t>8f41ef4a7f364268a627b36a96d66a3e</t>
+  </si>
+  <si>
+    <t>8ff8a31be76947ff989bd9121ee453be</t>
+  </si>
+  <si>
+    <t>903b062eb29943adae64c3dc685201b8</t>
+  </si>
+  <si>
+    <t>903da8e3807d42e794dcb11ef491e44c</t>
+  </si>
+  <si>
+    <t>909768e5e8bf4e72acffc822eb39398e</t>
+  </si>
+  <si>
+    <t>90ac783fffb642cf9f35c956ef34fed2</t>
+  </si>
+  <si>
+    <t>90f354376a7d47eab016dad56387e7f0</t>
+  </si>
+  <si>
+    <t>914367be62b14e129a74af0745dae03c</t>
+  </si>
+  <si>
+    <t>916c81b7604944dbad444ba04b3123fd</t>
+  </si>
+  <si>
+    <t>91b1a01acc3642a19bf7ca9c85707cab</t>
+  </si>
+  <si>
+    <t>91e97f20538840cf8d2c296bc9edf79b</t>
+  </si>
+  <si>
+    <t>9208daf7761a4e90ab3dce849269e804</t>
+  </si>
+  <si>
+    <t>9261604e232d437e90fb726029e6b971</t>
+  </si>
+  <si>
+    <t>92b5fc3846cb4cdea3544880ba5efbc6</t>
+  </si>
+  <si>
+    <t>92b9ba69a5ba4bf9b2700bf9b3158ab4</t>
+  </si>
+  <si>
+    <t>92c367f5bbb3401abc27559f2d94f9a5</t>
+  </si>
+  <si>
+    <t>93136bc377544cc1a2704995490e46d6</t>
+  </si>
+  <si>
+    <t>934a2d55b5f24f8bbccda35f22d97aaa</t>
+  </si>
+  <si>
+    <t>93f22b6a8991414e8acad1b3675e74ef</t>
+  </si>
+  <si>
+    <t>941f452f97324504b2cf3341c7d29bbd</t>
+  </si>
+  <si>
+    <t>9426bccd36ba4accb34433e1d9e8a1fe</t>
+  </si>
+  <si>
+    <t>943f3aa264544cdca7772848272badb3</t>
+  </si>
+  <si>
+    <t>94ce019a21ac42a68c4ab6646aa199ba</t>
+  </si>
+  <si>
+    <t>94e29dea4f2c4e35a1ba690ee7d0e471</t>
+  </si>
+  <si>
+    <t>959049cc858048609ee0a093bd1f13bf</t>
+  </si>
+  <si>
+    <t>95be396132004c4e8913688f6d5abf03</t>
+  </si>
+  <si>
+    <t>95c95b43cf3c435680df0aef2f33d83f</t>
+  </si>
+  <si>
+    <t>95dcd36548734b51bfff244c9ae507ff</t>
+  </si>
+  <si>
+    <t>95eb6f92038e441ba120b95058c34f38</t>
+  </si>
+  <si>
+    <t>95f3b2c6220140048a57bb7e4d90357f</t>
+  </si>
+  <si>
+    <t>96893b4bc80c4b0f8a8a33255b9ff2f8</t>
+  </si>
+  <si>
+    <t>96b90af74f6143d09a2926df0a573898</t>
+  </si>
+  <si>
+    <t>979864d9b21c49f2b2bdb2437a53724f</t>
+  </si>
+  <si>
+    <t>97e91d6b89dc44a58325bdaf67835544</t>
+  </si>
+  <si>
+    <t>98081d07dbf648b4936a2529c0e9e98d</t>
+  </si>
+  <si>
+    <t>981755f6b45340c0a3e2535f26aa9d1d</t>
+  </si>
+  <si>
+    <t>98a50b429b7d48a6a80e8d0a3c7c3d05</t>
+  </si>
+  <si>
+    <t>98da8d01657e4b7799e7b0fd6009a5e5</t>
+  </si>
+  <si>
+    <t>98eb6a3300ba4b709f95a87c741b33a3</t>
+  </si>
+  <si>
+    <t>99a75beb58f043789d87f3345ef8481a</t>
+  </si>
+  <si>
+    <t>99f6b6a6b082449ca36b62185e70cb86</t>
+  </si>
+  <si>
+    <t>9af1996fbe524b60aaf27f316a473fe1</t>
+  </si>
+  <si>
+    <t>9b3bcea7bf5e4822931f77991376e268</t>
+  </si>
+  <si>
+    <t>9b6d4e7f90a04330ab92bcdbc42327b3</t>
+  </si>
+  <si>
+    <t>9bc52e86c1304f20a8b291acdaca56e3</t>
+  </si>
+  <si>
+    <t>9c36a17f79894690bd625a802bcf2780</t>
+  </si>
+  <si>
+    <t>9d7032c937b14e05b6d0919bbee9bb8d</t>
+  </si>
+  <si>
+    <t>9da604e8b8cd4ecaa42c7372e41a36fe</t>
+  </si>
+  <si>
+    <t>9db478d2425548aeb978a518f9e2fcfd</t>
+  </si>
+  <si>
+    <t>9dd688f2336f4c42866e748e5c14e967</t>
+  </si>
+  <si>
+    <t>9e3ac4b4bae14ce5a10c9c3e3dca871c</t>
+  </si>
+  <si>
+    <t>9f169e51b4e746769d290dfe91f6b27d</t>
+  </si>
+  <si>
+    <t>9f5886c7d3934e51916d40508e238673</t>
+  </si>
+  <si>
+    <t>9f719c8036b44259bcd6efb1b81311bd</t>
+  </si>
+  <si>
+    <t>9fb73098f67e41e7a867e57d3eeee1a9</t>
+  </si>
+  <si>
+    <t>9fb80e8a9c5640b3a26c49ccc061ef75</t>
+  </si>
+  <si>
+    <t>a0355d2c84ec490f84f83df5a022e36a</t>
+  </si>
+  <si>
+    <t>a048f13e57c143cc91b4d261d372ceda</t>
+  </si>
+  <si>
+    <t>a050b179e77b4c69ab2ff9f4046139bd</t>
+  </si>
+  <si>
+    <t>a077a2cde3a24f9faa52816c70db28da</t>
+  </si>
+  <si>
+    <t>a0834aaa803e4b0aaa5a86f5bff0ee83</t>
+  </si>
+  <si>
+    <t>a0aa355e2718499c90ebe666456fd7c3</t>
+  </si>
+  <si>
+    <t>a0f7c6c3979c45ccaef7876b53125cc7</t>
+  </si>
+  <si>
+    <t>a10277a0ee144014b34d9f9c9b688ede</t>
+  </si>
+  <si>
+    <t>a151ed7575e24facbff10f412145dfdc</t>
+  </si>
+  <si>
+    <t>a187dfbe866748c1b857c189d5b6d1fe</t>
+  </si>
+  <si>
+    <t>a18e8b63c8694caaae36ee0bd46d5bcf</t>
+  </si>
+  <si>
+    <t>a1cedbecd3df4727bbcf35a2bb881c73</t>
+  </si>
+  <si>
+    <t>a1d450904e054ed0b1b6bed14aa113b6</t>
+  </si>
+  <si>
+    <t>a1e2b847c13f4e0fbea0bf136fbc459c</t>
+  </si>
+  <si>
+    <t>a1ebc590216e49199586d81721375ddf</t>
+  </si>
+  <si>
+    <t>a281fadb993f4ea08607bf4cc24ab4a7</t>
+  </si>
+  <si>
+    <t>a2e6cefeeb4b415b98896de61da9c395</t>
+  </si>
+  <si>
+    <t>a3bfed206636452a83979b92a87f7e77</t>
+  </si>
+  <si>
+    <t>a3c0c346de54449b900065d9f8fa1c46</t>
+  </si>
+  <si>
+    <t>a42390ec349b413f9455f8ffdf3dc03e</t>
+  </si>
+  <si>
+    <t>a4752a45e8a749b7b21640bbed59350a</t>
+  </si>
+  <si>
+    <t>a4bb5c2e8aec456ab360f6cfde8990a8</t>
+  </si>
+  <si>
+    <t>a4ece82b67474b5fb127ee7dbbfc13fb</t>
+  </si>
+  <si>
+    <t>a513a794a44241a0b333d0ce5d5fd998</t>
+  </si>
+  <si>
+    <t>a5ec9ade715b47bd9317a0ef1d2c7d7b</t>
+  </si>
+  <si>
+    <t>a5f17cd9b4374d57a7ee4fab41bbbf8e</t>
+  </si>
+  <si>
+    <t>a6102c0b18b24640a8e9b71ce05457d6</t>
+  </si>
+  <si>
+    <t>a62328977f5846228705a48f77559b18</t>
+  </si>
+  <si>
+    <t>a634cef020574d5b9aac0b2cc686bb13</t>
+  </si>
+  <si>
+    <t>a6b8f3a86abd4f77bebc002adf274fba</t>
+  </si>
+  <si>
+    <t>a6d36fdef32d4b66badbb774bc2a2261</t>
+  </si>
+  <si>
+    <t>a70a3043ba0249299b1ccbb159b44d4d</t>
+  </si>
+  <si>
+    <t>a72c69fbcee64be9bc986ad9faf82d50</t>
+  </si>
+  <si>
+    <t>a884ec13d7584b48a5ac5a1626a99fb8</t>
+  </si>
+  <si>
+    <t>a8d111276a684241b3b39c749ee6136a</t>
+  </si>
+  <si>
+    <t>a92e0bdfee07410a966ce2042d22f911</t>
+  </si>
+  <si>
+    <t>a957020c338943a5b4233b5c6f9226f0</t>
+  </si>
+  <si>
+    <t>a9b193bcbd6340529342385aabbffd6b</t>
+  </si>
+  <si>
+    <t>aa3922e2e84e4420a82e796e05f13836</t>
+  </si>
+  <si>
+    <t>aa3e55fe5f874f678fc16dd1eb16d07f</t>
+  </si>
+  <si>
+    <t>aa69520aaaa14fc48099643e246c7fd9</t>
+  </si>
+  <si>
+    <t>aad30f359ab840f39d72947c0c243020</t>
+  </si>
+  <si>
+    <t>ab171cb8b1124291b3ef5571eee00d9f</t>
+  </si>
+  <si>
+    <t>ac22c7dc0cc24e22be56fbee7a589208</t>
+  </si>
+  <si>
+    <t>ac2ba1e100cb44e0b69e08c78f7dfefe</t>
+  </si>
+  <si>
+    <t>ac894f4ba31740a5a1b61ecea9ae2963</t>
+  </si>
+  <si>
+    <t>aca7ce041d294b2d9e2d6b713e6ada37</t>
+  </si>
+  <si>
+    <t>acc14373283547b59fc586662899c0c6</t>
+  </si>
+  <si>
+    <t>acda636c3c11482493d0d32cc01c95da</t>
+  </si>
+  <si>
+    <t>acfbb1d066f9403dbd3e013a6220a854</t>
+  </si>
+  <si>
+    <t>ad5bfc8f368844c8853f41371be1a088</t>
+  </si>
+  <si>
+    <t>ad6f240bdedf42b586722cd4a4ca7d92</t>
+  </si>
+  <si>
+    <t>ad8a752be4204f87a7b354b9822e6779</t>
+  </si>
+  <si>
+    <t>ae80d8d832a9420baac58bfcb6bbdb28</t>
+  </si>
+  <si>
+    <t>ae9c7cc42e3d4b799d4ad9b15e98a719</t>
+  </si>
+  <si>
+    <t>aeaeef67b61e42b2a7fdda4556237d92</t>
+  </si>
+  <si>
+    <t>aeb48fae40614dcca8f234f5f5e4b497</t>
+  </si>
+  <si>
+    <t>afa4c18543f5404ab4dbeaaea383dbf7</t>
+  </si>
+  <si>
+    <t>afd01779d3b9450ca4d131a4423ad9f5</t>
+  </si>
+  <si>
+    <t>b011a514f1714d21a0afab7a331d0a59</t>
+  </si>
+  <si>
+    <t>b082a84b766e4c58b6914d49f09db48e</t>
+  </si>
+  <si>
+    <t>b0e8673bae284a4eb49f076a09edc399</t>
+  </si>
+  <si>
+    <t>b12fc5ebf5704129ad6cc5a8408b6892</t>
+  </si>
+  <si>
+    <t>b164702b6d82483f9faa76987109ee21</t>
+  </si>
+  <si>
+    <t>b20f6cf317eb422b9e53ff121ce69117</t>
+  </si>
+  <si>
+    <t>b284c65605c74139964c8e3e0ab55f11</t>
+  </si>
+  <si>
+    <t>b2dc9d621be64d9a8cf5ae2652cec05c</t>
+  </si>
+  <si>
+    <t>b3058fa8f020461fa6bdd97fcffaa10f</t>
+  </si>
+  <si>
+    <t>b33fa6c348fd448c846286cfeb9614de</t>
+  </si>
+  <si>
+    <t>b352442c5016494cbe3a29a6c5a54eba</t>
+  </si>
+  <si>
+    <t>b3d78e8ac6ea4deabdc53521d563194a</t>
+  </si>
+  <si>
+    <t>b4173093104c4721bfa9e66352bcc456</t>
+  </si>
+  <si>
+    <t>b45c775e93954118ab18d0352ebd50b4</t>
+  </si>
+  <si>
+    <t>b54adc17ea004d5cb7e0d4a501df67a4</t>
+  </si>
+  <si>
+    <t>b64e265f196041ce9e32ba807f57f908</t>
+  </si>
+  <si>
+    <t>b666e95e47464635952ec5be0e42b625</t>
+  </si>
+  <si>
+    <t>b695ca6ca8a24c7abc24004483afe394</t>
+  </si>
+  <si>
+    <t>b6dee6cdc00f46d9a25ac51e666999da</t>
+  </si>
+  <si>
+    <t>b6e3eca2ae384954b65bc05bb882df7b</t>
+  </si>
+  <si>
+    <t>b6e970975be04c69a5de66907a058190</t>
+  </si>
+  <si>
+    <t>b7cd8bf81d564e8e8ec72bf3800a6e1a</t>
+  </si>
+  <si>
+    <t>b80f6717f1154fff8503dce14f1579f8</t>
+  </si>
+  <si>
+    <t>b8528a3197b34713a75bf9d69768bfc9</t>
+  </si>
+  <si>
+    <t>b8cbb4bc93e746df9cd0b2d02ec3f695</t>
+  </si>
+  <si>
+    <t>b90efd28547e410e94375107c59ca4b0</t>
+  </si>
+  <si>
+    <t>b946847b03744360bac114dae8bdeba0</t>
+  </si>
+  <si>
+    <t>b986733ea5b84958a55117726cf1a613</t>
+  </si>
+  <si>
+    <t>b9e9ca2290e94ef9992a73e3e92ef6cb</t>
+  </si>
+  <si>
+    <t>ba3d963a17fa472cb1e5b4588dfdadda</t>
+  </si>
+  <si>
+    <t>bb301458149347f8b87632bf0b0c5da4</t>
+  </si>
+  <si>
+    <t>bbd0ff5a98db4b38951b41b3737da054</t>
+  </si>
+  <si>
+    <t>bbfc5aa41aab431f941ffa09a72ab922</t>
+  </si>
+  <si>
+    <t>bc17086e48d347efb315b134311133a3</t>
+  </si>
+  <si>
+    <t>bc7b7265d9054a45ba543e1566ab988a</t>
+  </si>
+  <si>
+    <t>bd20cb3c03be42ed901a08613ccf23f1</t>
+  </si>
+  <si>
+    <t>bd7f88f29bc74339b3163b639584737d</t>
+  </si>
+  <si>
+    <t>be3e084bc4ca4e7db69b04deaa3dee00</t>
+  </si>
+  <si>
+    <t>be5ffa6ee9994cbcbb671da3d8d50fdf</t>
+  </si>
+  <si>
+    <t>be8ecbf300d941cc8639ebb913d26f83</t>
+  </si>
+  <si>
+    <t>bf1fd60860ff405689997a5546c91bea</t>
+  </si>
+  <si>
+    <t>bff928df38a6439491f600a5a4af8569</t>
+  </si>
+  <si>
+    <t>c0715828c3494be5a3eb3177b9065296</t>
+  </si>
+  <si>
+    <t>c0992296fb294eb8b9e60480144c737d</t>
+  </si>
+  <si>
+    <t>c1400abeb6064621a742290ac5f7d05d</t>
+  </si>
+  <si>
+    <t>c16007074b8144b897a82740a5736de3</t>
+  </si>
+  <si>
+    <t>c16810aca9fc4864af94011a3af7aa9a</t>
+  </si>
+  <si>
+    <t>c17c6804511b43ef873620137c5a8d23</t>
+  </si>
+  <si>
+    <t>c17c7f63429e43a199c82d3e9e130404</t>
+  </si>
+  <si>
+    <t>c1c28789aafb4924a59cf088f65725ab</t>
+  </si>
+  <si>
+    <t>c24ab6cec9e349cb8adc7bc7989c5714</t>
+  </si>
+  <si>
+    <t>c25527a5b40a4c4691738199efdbb027</t>
+  </si>
+  <si>
+    <t>c26a00ce04014308803dfeacd0f9ea84</t>
+  </si>
+  <si>
+    <t>c30733060779410d9e6fae63bf0d0e0e</t>
+  </si>
+  <si>
+    <t>c3147a77a8e34766933a0d9c88e99d56</t>
+  </si>
+  <si>
+    <t>c32781387a9b4010b88e3dd8b4bef8c5</t>
+  </si>
+  <si>
+    <t>c32d759979e04cfab401a9b139973ee5</t>
+  </si>
+  <si>
+    <t>c3309dbd52374d7995f932e7d40b6876</t>
+  </si>
+  <si>
+    <t>c3ff970dddf340c6b16f3e8145cf69d4</t>
+  </si>
+  <si>
+    <t>c41f193ed3e2480f8e363391e1c8cf53</t>
+  </si>
+  <si>
+    <t>c558873efc604c9a9fb12cff95d1690a</t>
+  </si>
+  <si>
+    <t>c5cf860108e34932aef2fd637c81042b</t>
+  </si>
+  <si>
+    <t>c608bea5bfad45d496fc66b6189e33e6</t>
+  </si>
+  <si>
+    <t>c657f85f61df48a8af5083177de0b9e0</t>
+  </si>
+  <si>
+    <t>c66ac54303b849d98c980211297cb4e4</t>
+  </si>
+  <si>
+    <t>c6ac859a0a52458db08d3d7de116735d</t>
+  </si>
+  <si>
+    <t>c7278cd526a24c7cbeb9577ca2a8be0a</t>
+  </si>
+  <si>
+    <t>c7958897f22d41e89fe7f74dd825e5b3</t>
+  </si>
+  <si>
+    <t>c8713e31ea3f4fd7849290e66757f148</t>
+  </si>
+  <si>
+    <t>c8b9e44181e444b6b7bcde8609d0076a</t>
+  </si>
+  <si>
+    <t>c93f91b5675646acaa972fbc0c0ece79</t>
+  </si>
+  <si>
+    <t>ca81b4728c424ccf9dac2deac7b670f5</t>
+  </si>
+  <si>
+    <t>cab1c632261e44c784acebb65ea8f7ea</t>
+  </si>
+  <si>
+    <t>cad254373fc140f989fc79674acc504c</t>
+  </si>
+  <si>
+    <t>cbda0f31d98a4851a0dc56b4871b16f7</t>
+  </si>
+  <si>
+    <t>cbf0a4cd0baf4021aa7db1a0cfe97287</t>
+  </si>
+  <si>
+    <t>cccffd6c272d4cee8acc1a1885acf077</t>
+  </si>
+  <si>
+    <t>cce0256a65b242c7806d861ae4905516</t>
+  </si>
+  <si>
+    <t>cd31e2eff4634e79aaf8457421174ecb</t>
+  </si>
+  <si>
+    <t>cd737f5b31e04690af021a1af990d8a9</t>
+  </si>
+  <si>
+    <t>cdd946e78b2d478c8c7fccdd2e44df75</t>
+  </si>
+  <si>
+    <t>cec681c0c027469eb5c6b0db9c48482f</t>
+  </si>
+  <si>
+    <t>cefd48e4f7e44888bbc98ece1b122215</t>
+  </si>
+  <si>
+    <t>cf75697757fa4f37ac883e6a7bfcf938</t>
+  </si>
+  <si>
+    <t>cf949ec95e5243eb997c514bf953e01c</t>
+  </si>
+  <si>
+    <t>d087612b5f1b437ba2e0fb5c4cdc0cb1</t>
+  </si>
+  <si>
+    <t>d0ee91666e244420a265180feba5a956</t>
+  </si>
+  <si>
+    <t>d18e9732a3324ac09fb1d1d074ff1dee</t>
+  </si>
+  <si>
+    <t>d1957a08ebbb46e9a4fa27c98c95be2b</t>
+  </si>
+  <si>
+    <t>d19c40208b6d41d5897e912ef02f93ec</t>
+  </si>
+  <si>
+    <t>d225f7d2624148cd9f88ca8eb061f42e</t>
+  </si>
+  <si>
+    <t>d265b67d3d3f4f22b2167e9722f46fc9</t>
+  </si>
+  <si>
+    <t>d2a23785dc814c1eab254795b24ab45a</t>
+  </si>
+  <si>
+    <t>d3165771c8914e09af8472a49a81c8f6</t>
+  </si>
+  <si>
+    <t>d387b094797647e39f612a76e93678f0</t>
+  </si>
+  <si>
+    <t>d3ef84eb631845c58d71df4ba526bab4</t>
+  </si>
+  <si>
+    <t>d420f07f64534237b560bc6837bc67e0</t>
+  </si>
+  <si>
+    <t>d4a8d0f8e7b347049788c31f359faeb4</t>
+  </si>
+  <si>
+    <t>d4bce10efb224d029dd2489a0d1c71d9</t>
+  </si>
+  <si>
+    <t>d558f9553aa24d7ab3f7854a2f93b706</t>
+  </si>
+  <si>
+    <t>d5b261a910234f18ba7723b3a6dfa584</t>
+  </si>
+  <si>
+    <t>d5f5d4491cf94265b1834c713e4ce574</t>
+  </si>
+  <si>
+    <t>d605d762829943f0908d167a4cdc4c6f</t>
+  </si>
+  <si>
+    <t>d6b95aabc6664af4988bb5cae1c3f819</t>
+  </si>
+  <si>
+    <t>d8bc65978f2c4770bc6498317a4e3046</t>
+  </si>
+  <si>
+    <t>d91564cbb64c46308db74f029f437c11</t>
+  </si>
+  <si>
+    <t>d92c3f3dcba4446db666f3826f7cde7e</t>
+  </si>
+  <si>
+    <t>d9c51f5bde634437beeed4e9def982c3</t>
+  </si>
+  <si>
+    <t>da74ef68b8e04c7bb854a76a7d09d2b9</t>
+  </si>
+  <si>
+    <t>dab57a3aee874592b609dd1f39eb4f3d</t>
+  </si>
+  <si>
+    <t>dac66e67f5a4443691836c46ed8fe3a7</t>
+  </si>
+  <si>
+    <t>db2aa492c4f34fa898c80e5cc3ccef68</t>
+  </si>
+  <si>
+    <t>dc0dbcdc526143c2b022c33447cec358</t>
+  </si>
+  <si>
+    <t>dc16f498ff444da2a8e7fb81f085f796</t>
+  </si>
+  <si>
+    <t>dc1bb2d8cfc0465d9c96a512078393e5</t>
+  </si>
+  <si>
+    <t>dcb3c12840014c60acdd3eb6a4132d6f</t>
+  </si>
+  <si>
+    <t>dcbfa71740464aa8b0306a6f9544d24d</t>
+  </si>
+  <si>
+    <t>dd0f6e2b6c6a46fda9f4ec152b606296</t>
+  </si>
+  <si>
+    <t>dd9b2354c8cb4c44b27f85a0fc5057d5</t>
+  </si>
+  <si>
+    <t>ddf83fc4785649e7a5758c7b9238c7bc</t>
+  </si>
+  <si>
+    <t>de77e681355e48889ce780784ced0b58</t>
+  </si>
+  <si>
+    <t>de990baa5e564a16b07cab88596776bf</t>
+  </si>
+  <si>
+    <t>df188cf3af7a43beaf163ba4a975647d</t>
+  </si>
+  <si>
+    <t>df193bae2cb543619a86aa79f47b9adc</t>
+  </si>
+  <si>
+    <t>df78ae76a3a644c7b1c08f7c710f0300</t>
+  </si>
+  <si>
+    <t>df7abf0b86b7431d9c1a0a72aa273075</t>
+  </si>
+  <si>
+    <t>dfb876dd895146998bda3ced43da4007</t>
+  </si>
+  <si>
+    <t>dfd0aea0b8d1413386d59269bca77523</t>
+  </si>
+  <si>
+    <t>e016a146ca7142d88cb0e831350d5916</t>
+  </si>
+  <si>
+    <t>e02b55c638f8486c9b4258d2f8bbdbd0</t>
+  </si>
+  <si>
+    <t>e10f2dd34ee04932882203ced875fcb7</t>
+  </si>
+  <si>
+    <t>e222acc59895458da20c652221fb2e1e</t>
+  </si>
+  <si>
+    <t>e24c3de5562c4a9da3cd740798fe4feb</t>
+  </si>
+  <si>
+    <t>e261aa7a910c43bea28f32aef75a893b</t>
+  </si>
+  <si>
+    <t>e3224742268244a987983b0bcaa5eb3b</t>
+  </si>
+  <si>
+    <t>e347e0db8d6241e0a2657e9de1daf365</t>
+  </si>
+  <si>
+    <t>e3998e079f9947549762aa9e22adf8ac</t>
+  </si>
+  <si>
+    <t>e49970eacfb64bfaa5ba28e60bc09f5b</t>
+  </si>
+  <si>
+    <t>e4b268eb0e19463f8e8be4dd05037fa2</t>
+  </si>
+  <si>
+    <t>e4bec82c2e1f46339f94c8a6f7d10d76</t>
+  </si>
+  <si>
+    <t>e50c563ab6af4415a017fbcf46b90440</t>
+  </si>
+  <si>
+    <t>e57662b9278a4495898bc3cfe6f94ba5</t>
+  </si>
+  <si>
+    <t>e582deb9d9e74b87aeb4d439e09ac221</t>
+  </si>
+  <si>
+    <t>e5881e901fa1499dae608ffec28aaa47</t>
+  </si>
+  <si>
+    <t>e5ae796a0b804f28a6e96ec5545ddf9f</t>
+  </si>
+  <si>
+    <t>e5f914ebd1ec499894b34593d9e838de</t>
+  </si>
+  <si>
+    <t>e6928620e0684bd082fcf0ffb825b018</t>
+  </si>
+  <si>
+    <t>e6d9aefb820e43aba4b6ebbc4a8e4b44</t>
+  </si>
+  <si>
+    <t>e6eb3c1e6f8e472e911a47a38938fa36</t>
+  </si>
+  <si>
+    <t>e7c89783610445029d58ecd383defd35</t>
+  </si>
+  <si>
+    <t>e8115e5732ca4fbbac9c2785cd48549b</t>
+  </si>
+  <si>
+    <t>e85d610b9075486ca3f0edd437ee9da6</t>
+  </si>
+  <si>
+    <t>e87cf47ced7548f086e1acd713436109</t>
+  </si>
+  <si>
+    <t>e88168f8c5e843b3b228716c64edae90</t>
+  </si>
+  <si>
+    <t>e8f4f37cbab64576910c5a6074ec0aec</t>
+  </si>
+  <si>
+    <t>e909e22f695640a3ae64a651a762ef42</t>
+  </si>
+  <si>
+    <t>e9690650f1484e7792e809bafea10944</t>
+  </si>
+  <si>
+    <t>e9b3f6219c024922822523c8a32a83ec</t>
+  </si>
+  <si>
+    <t>ea234d67731646cd9eb5a217bd3f3ad1</t>
+  </si>
+  <si>
+    <t>ea6fb0f25f1c4ef19113435e4bde7898</t>
+  </si>
+  <si>
+    <t>ea92dd1c51624ecc88d15ad043303099</t>
+  </si>
+  <si>
+    <t>eb228a31426d4597b9fe2c58b9d12ebe</t>
+  </si>
+  <si>
+    <t>eb5ccd3a62684b2185eb96bde7b9d9b6</t>
+  </si>
+  <si>
+    <t>eb7c774b989a4c8083865e5de9a7f646</t>
+  </si>
+  <si>
+    <t>ebcb62bd86fd4a758ff0c2f442cbc668</t>
+  </si>
+  <si>
+    <t>ebe9c4cd58a84a41a2e03fde7dde7fce</t>
+  </si>
+  <si>
+    <t>ebf1c0f8c57b427db96ab6c23cf8277a</t>
+  </si>
+  <si>
+    <t>ec005b1ac5cf4cc19c4662bcc19bcb9b</t>
+  </si>
+  <si>
+    <t>ec2c7f786fc14d6d8d3df6aaef3a7820</t>
+  </si>
+  <si>
+    <t>ec33cd95b22b4432b711d43cf3a5b4cd</t>
+  </si>
+  <si>
+    <t>ec9aa2448c4e43e3b3d0d06cc35d2537</t>
+  </si>
+  <si>
+    <t>ece07174d36c48f5aa6e7ea5855e6d79</t>
+  </si>
+  <si>
+    <t>ecf9d31ff3484409b1897425633f6b45</t>
+  </si>
+  <si>
+    <t>ee165adae53d425f954bde33f5693edd</t>
+  </si>
+  <si>
+    <t>eee119e06816429cafd3c9f5ec576b96</t>
+  </si>
+  <si>
+    <t>efe17beabc784c36a97bae435f56faca</t>
+  </si>
+  <si>
+    <t>f0290f34e0ea49019c4bb67897ee0294</t>
+  </si>
+  <si>
+    <t>f04c688e52df460992254d079f378801</t>
+  </si>
+  <si>
+    <t>f06bead7f5544d009eefad5bf3273932</t>
+  </si>
+  <si>
+    <t>f079558fb4d64ba2ba8b8d9e1c5d3809</t>
+  </si>
+  <si>
+    <t>f103a79a148c4b44beb94c2eeb2088db</t>
+  </si>
+  <si>
+    <t>f11e5021c7d44fb1b92875f5a72ccad0</t>
+  </si>
+  <si>
+    <t>f15d99d8343d4b8ca726e33d6e9dd2cc</t>
+  </si>
+  <si>
+    <t>f1e94fd8b6e549a787d62c774ec64725</t>
+  </si>
+  <si>
+    <t>f2704103dd98408ab6d24e3214a6e752</t>
+  </si>
+  <si>
+    <t>f2bb35f46e79443c84046fa93bd1e207</t>
+  </si>
+  <si>
+    <t>f3af260b8c8e409984ca759f85d33919</t>
+  </si>
+  <si>
+    <t>f3d7f340ab034853b7c6b7049c95408c</t>
+  </si>
+  <si>
+    <t>f44ec64a6f464ba896212e0daa3e391b</t>
+  </si>
+  <si>
+    <t>f49b1e3c9c324d37b80be2ff57078071</t>
+  </si>
+  <si>
+    <t>f4bf6bc18cde4e09ae6e222231702bdd</t>
+  </si>
+  <si>
+    <t>f514052dc6da4e14a208829f69ede874</t>
+  </si>
+  <si>
+    <t>f56c48f0f2444d67bb4fe214a93b1c85</t>
+  </si>
+  <si>
+    <t>f589daf42d974ae6ba3300cb941e8db6</t>
+  </si>
+  <si>
+    <t>f5df7a10186f4a21853e5e862a26cff0</t>
+  </si>
+  <si>
+    <t>f5ed401a077747bcaae233350cc56bb8</t>
+  </si>
+  <si>
+    <t>f6141c38e6ea4af8b9531ba5bff89dd5</t>
+  </si>
+  <si>
+    <t>f64d2a9cf1a7487fade1ea023178fe8c</t>
+  </si>
+  <si>
+    <t>f65cfadfb1df4d5996d8a4c401e3ccf0</t>
+  </si>
+  <si>
+    <t>f6734d24abed4eeeaf0b70200ef37ede</t>
+  </si>
+  <si>
+    <t>f6ac4f67ae994e43bb7eba9387ca14d8</t>
+  </si>
+  <si>
+    <t>f6cf11322ba5457ab0d8f1a252c1b21d</t>
+  </si>
+  <si>
+    <t>f6d3b5d857774c83ba0302e7dae00364</t>
+  </si>
+  <si>
+    <t>f6d808371f2243e08af170490fb52c90</t>
+  </si>
+  <si>
+    <t>f70524384e354d57bd8e317d28e362de</t>
+  </si>
+  <si>
+    <t>f70d2e2a09c4429bb9c83fa999977e60</t>
+  </si>
+  <si>
+    <t>f73ceb80b3ce41e8acf92b440249cfdb</t>
+  </si>
+  <si>
+    <t>f78e700dfa8d43dab9a8e73544550b8a</t>
+  </si>
+  <si>
+    <t>f828243477794a4ca6f486ce23e20ab1</t>
+  </si>
+  <si>
+    <t>f9515a78b62746ce969137d50fbaa96d</t>
+  </si>
+  <si>
+    <t>f95c7ba943744f60a220a63662ba4998</t>
+  </si>
+  <si>
+    <t>f96d5058824b4ba4966a19a856d9816f</t>
+  </si>
+  <si>
+    <t>fa060e4606ef407ea4d70154088d9e61</t>
+  </si>
+  <si>
+    <t>fa48174672884b108d043e000062a2c1</t>
+  </si>
+  <si>
+    <t>faf089ed71ec4f79a0b5bb47532a0b5c</t>
+  </si>
+  <si>
+    <t>fb8cd1177cdf471395a79bb206084319</t>
+  </si>
+  <si>
+    <t>fbb4a19691294dbabb2d86c33281f9c9</t>
+  </si>
+  <si>
+    <t>fc5727ca159a4042b7a138f853d5217c</t>
+  </si>
+  <si>
+    <t>fc633d027ace415eb43176a0860ac510</t>
+  </si>
+  <si>
+    <t>fcaebff3228648c6b884b46545b62684</t>
+  </si>
+  <si>
+    <t>fcdb4659958c41e3b9fcfa64cb366470</t>
+  </si>
+  <si>
+    <t>fd5894bd35e14c9db08ca6bb47bf82b9</t>
+  </si>
+  <si>
+    <t>fd603d97740e4a9c8228aebd26480749</t>
+  </si>
+  <si>
+    <t>fdab8165b491466ea5cb1cc5d9408bf7</t>
+  </si>
+  <si>
+    <t>fdd1b6e233e44eddadb49802218fb302</t>
+  </si>
+  <si>
+    <t>fdd670b18915449dadfd20a032fb1752</t>
+  </si>
+  <si>
+    <t>fe2c98c422f3437a9f0370076db8c5af</t>
+  </si>
+  <si>
+    <t>fe7f7af51ea94b04a9bf2627093a36e0</t>
+  </si>
+  <si>
+    <t>fe901a793718481babd2b6025e6bf0ce</t>
+  </si>
+  <si>
+    <t>feb34cbd850042d4aa3d836d48a4131d</t>
+  </si>
+  <si>
+    <t>fec4dbd90b6e4389b44971bd08b7e072</t>
+  </si>
+  <si>
+    <t>ff2b614a084244cba930b5cac5a54375</t>
+  </si>
+  <si>
+    <t>ff2ef148c80845b4a8ed0146762957a3</t>
+  </si>
+  <si>
+    <t>ff7714a7aa6b44b9ab04dbd98aeb4ce3</t>
+  </si>
+  <si>
+    <t>ffafa3c2cacc43cfae94059840315953</t>
+  </si>
+  <si>
+    <t>ffe505fde17f4a609b607e49a22684cc</t>
+  </si>
+  <si>
+    <t>fff3ecf2bcad4d5bb5b0b180f98ad500</t>
+  </si>
+  <si>
+    <t>fffb73f2b4e24bd7909e108bf76c20d9</t>
   </si>
 </sst>
 </file>

</xml_diff>